<commit_message>
Jahresplanung: roter Heute-Rahmen, Vorlauf aus dem Gantt
- Heute-Rahmen rot und lückenlos; keine bedingten Rahmen mehr auf
  verbundenen Teilzellen (Wochentagszeile zentriert über Auswahl)
- Standard-Vorläufe oben entfernt; Vorlauf Sommer-/Weihnachtsmailing
  wird aus dem Gantt (Blatt 2/3) übernommen, übrige Maßnahmen individuell
- Gantt wieder rückwärts vom PAL mit festen Dauern; Prüfanzeige
  "Zeitplan ok" entfernt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Efpubc9TCkNCWzy5pGdKJy
</commit_message>
<xml_diff>
--- a/excel/260924_Jahresplanung_Aussenkommunikation_2027_MA.xlsx
+++ b/excel/260924_Jahresplanung_Aussenkommunikation_2027_MA.xlsx
@@ -33,8 +33,6 @@
     <definedName name="Projekt_Start" localSheetId="2">Weihnachtsmailing!$C$6</definedName>
     <definedName name="Scroll_Schrittweite" localSheetId="1">Sommermailing!$C$7</definedName>
     <definedName name="Scroll_Schrittweite" localSheetId="2">Weihnachtsmailing!$C$7</definedName>
-    <definedName name="Std_Vorlauf_Inhalt">Jahresplanung!$W$6</definedName>
-    <definedName name="Std_Vorlauf_Sel">Jahresplanung!$W$5</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -57,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="154">
   <si>
     <t xml:space="preserve">Erstellen eines Gantt-Diagramms
 Geben Sie den Titel dieses Projekts in Zelle B2 ein.
@@ -584,6 +582,12 @@
   </si>
   <si>
     <t>Bußgeldmailing 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vorlauf: Bei Sommer- und Weihnachtsmailing wird er automatisch aus dem Gantt übernommen (Summe der Arbeitsschritte bis zum PAL, graue Felder). Bei allen anderen Maßnahmen individuell eintragen; Zelle leeren = kein Termin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sommer- und Weihnachtsmailing: Der PAL hier steuert die gleichnamigen Detailblätter. Dauern der Arbeitsschritte im Gantt ändern = Vorlauf und Starttermine hier ändern sich mit. Verknüpfung über den Namen in Spalte „Maßnahme“.</t>
   </si>
 </sst>
 </file>
@@ -1887,7 +1891,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="191">
+  <cellXfs count="198">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2439,6 +2443,27 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="1" fontId="66" fillId="20" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="66" fillId="20" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="66" fillId="20" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="66" fillId="20" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Akzent3" xfId="11" builtinId="37"/>
@@ -2454,7 +2479,7 @@
     <cellStyle name="Überschrift 3" xfId="8" builtinId="18" customBuiltin="1"/>
     <cellStyle name="zAusgeblText" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="136">
+  <dxfs count="142">
     <dxf>
       <font>
         <i/>
@@ -3912,6 +3937,57 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <border>
+        <left style="thin">
+          <color rgb="FFE30714"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color rgb="FFE30714"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FFE30714"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FFE30714"/>
+        </left>
+        <bottom style="thin">
+          <color rgb="FFE30714"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color rgb="FFE30714"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <right style="thin">
+          <color rgb="FFE30714"/>
+        </right>
+        <bottom style="thin">
+          <color rgb="FFE30714"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Gantt-Tabellenformat" pivot="0" count="4" xr9:uid="{4904D139-63E4-4221-B7C9-C6C5B7A50FAF}">
@@ -4794,36 +4870,6 @@
       <c r="CN4" s="121"/>
     </row>
     <row r="5" spans="2:92" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="116" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" s="116"/>
-      <c r="D5" s="116"/>
-      <c r="E5" s="116"/>
-      <c r="F5" s="116"/>
-      <c r="G5" s="116"/>
-      <c r="H5" s="116"/>
-      <c r="I5" s="116"/>
-      <c r="J5" s="116"/>
-      <c r="K5" s="116"/>
-      <c r="L5" s="116"/>
-      <c r="M5" s="116"/>
-      <c r="N5" s="116"/>
-      <c r="O5" s="116"/>
-      <c r="P5" s="116"/>
-      <c r="Q5" s="116"/>
-      <c r="R5" s="116"/>
-      <c r="S5" s="116"/>
-      <c r="T5" s="116"/>
-      <c r="U5" s="116"/>
-      <c r="V5" s="116"/>
-      <c r="W5" s="117">
-        <v>76</v>
-      </c>
-      <c r="X5" s="118"/>
-      <c r="Y5" s="118"/>
-      <c r="Z5" s="118"/>
-      <c r="AA5" s="118"/>
       <c r="AE5" s="116" t="s">
         <v>61</v>
       </c>
@@ -4891,36 +4937,6 @@
       <c r="CN5" s="121"/>
     </row>
     <row r="6" spans="2:92" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="116" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="116"/>
-      <c r="D6" s="116"/>
-      <c r="E6" s="116"/>
-      <c r="F6" s="116"/>
-      <c r="G6" s="116"/>
-      <c r="H6" s="116"/>
-      <c r="I6" s="116"/>
-      <c r="J6" s="116"/>
-      <c r="K6" s="116"/>
-      <c r="L6" s="116"/>
-      <c r="M6" s="116"/>
-      <c r="N6" s="116"/>
-      <c r="O6" s="116"/>
-      <c r="P6" s="116"/>
-      <c r="Q6" s="116"/>
-      <c r="R6" s="116"/>
-      <c r="S6" s="116"/>
-      <c r="T6" s="116"/>
-      <c r="U6" s="116"/>
-      <c r="V6" s="116"/>
-      <c r="W6" s="117">
-        <v>58</v>
-      </c>
-      <c r="X6" s="118"/>
-      <c r="Y6" s="118"/>
-      <c r="Z6" s="118"/>
-      <c r="AA6" s="118"/>
       <c r="AE6" s="116" t="s">
         <v>65</v>
       </c>
@@ -5016,10 +5032,7 @@
       <c r="AA7" s="119"/>
       <c r="AB7" s="119"/>
       <c r="AC7" s="119"/>
-      <c r="AE7" s="120" t="str">
-        <f>IF(AND(Sommermailing!$G$14&gt;=1,Sommermailing!$G$17&gt;=1),"✓ Sommermailing: Zeitplan ok","⚠ Sommermailing: Vorlauf zu kurz")</f>
-        <v>✓ Sommermailing: Zeitplan ok</v>
-      </c>
+      <c r="AE7" s="120"/>
       <c r="AF7" s="120"/>
       <c r="AG7" s="120"/>
       <c r="AH7" s="120"/>
@@ -5037,10 +5050,7 @@
       <c r="AT7" s="120"/>
       <c r="AU7" s="120"/>
       <c r="AV7" s="120"/>
-      <c r="AX7" s="120" t="str">
-        <f>IF(AND(Weihnachtsmailing!$G$14&gt;=1,Weihnachtsmailing!$G$17&gt;=1),"✓ Weihnachtsmailing: Zeitplan ok","⚠ Weihnachtsmailing: Vorlauf zu kurz")</f>
-        <v>✓ Weihnachtsmailing: Zeitplan ok</v>
-      </c>
+      <c r="AX7" s="120"/>
       <c r="AY7" s="120"/>
       <c r="AZ7" s="120"/>
       <c r="BA7" s="120"/>
@@ -5292,155 +5302,155 @@
       <c r="B12" s="163" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="124" t="s">
+      <c r="C12" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="124"/>
-      <c r="E12" s="124"/>
-      <c r="F12" s="124" t="s">
+      <c r="D12" s="191"/>
+      <c r="E12" s="191"/>
+      <c r="F12" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="G12" s="124"/>
-      <c r="H12" s="124"/>
-      <c r="I12" s="124" t="s">
+      <c r="G12" s="191"/>
+      <c r="H12" s="191"/>
+      <c r="I12" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="J12" s="124"/>
-      <c r="K12" s="124"/>
-      <c r="L12" s="124" t="s">
+      <c r="J12" s="191"/>
+      <c r="K12" s="191"/>
+      <c r="L12" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="M12" s="124"/>
-      <c r="N12" s="124"/>
-      <c r="O12" s="124" t="s">
+      <c r="M12" s="191"/>
+      <c r="N12" s="191"/>
+      <c r="O12" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="P12" s="124"/>
-      <c r="Q12" s="124"/>
-      <c r="R12" s="124" t="s">
+      <c r="P12" s="191"/>
+      <c r="Q12" s="191"/>
+      <c r="R12" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="S12" s="124"/>
-      <c r="T12" s="124"/>
-      <c r="U12" s="124" t="s">
+      <c r="S12" s="191"/>
+      <c r="T12" s="191"/>
+      <c r="U12" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="V12" s="124"/>
-      <c r="W12" s="164"/>
+      <c r="V12" s="191"/>
+      <c r="W12" s="192"/>
       <c r="Y12" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="Z12" s="124" t="s">
+      <c r="Z12" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="AA12" s="124"/>
-      <c r="AB12" s="124"/>
-      <c r="AC12" s="124" t="s">
+      <c r="AA12" s="191"/>
+      <c r="AB12" s="191"/>
+      <c r="AC12" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="AD12" s="124"/>
-      <c r="AE12" s="124"/>
-      <c r="AF12" s="124" t="s">
+      <c r="AD12" s="191"/>
+      <c r="AE12" s="191"/>
+      <c r="AF12" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="AG12" s="124"/>
-      <c r="AH12" s="124"/>
-      <c r="AI12" s="124" t="s">
+      <c r="AG12" s="191"/>
+      <c r="AH12" s="191"/>
+      <c r="AI12" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="AJ12" s="124"/>
-      <c r="AK12" s="124"/>
-      <c r="AL12" s="124" t="s">
+      <c r="AJ12" s="191"/>
+      <c r="AK12" s="191"/>
+      <c r="AL12" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="AM12" s="124"/>
-      <c r="AN12" s="124"/>
-      <c r="AO12" s="124" t="s">
+      <c r="AM12" s="191"/>
+      <c r="AN12" s="191"/>
+      <c r="AO12" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="AP12" s="124"/>
-      <c r="AQ12" s="124"/>
-      <c r="AR12" s="124" t="s">
+      <c r="AP12" s="191"/>
+      <c r="AQ12" s="191"/>
+      <c r="AR12" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="AS12" s="124"/>
-      <c r="AT12" s="176"/>
+      <c r="AS12" s="191"/>
+      <c r="AT12" s="193"/>
       <c r="AV12" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="AW12" s="124" t="s">
+      <c r="AW12" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="AX12" s="124"/>
-      <c r="AY12" s="124"/>
-      <c r="AZ12" s="124" t="s">
+      <c r="AX12" s="191"/>
+      <c r="AY12" s="191"/>
+      <c r="AZ12" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="BA12" s="124"/>
-      <c r="BB12" s="124"/>
-      <c r="BC12" s="124" t="s">
+      <c r="BA12" s="191"/>
+      <c r="BB12" s="191"/>
+      <c r="BC12" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="BD12" s="124"/>
-      <c r="BE12" s="124"/>
-      <c r="BF12" s="124" t="s">
+      <c r="BD12" s="191"/>
+      <c r="BE12" s="191"/>
+      <c r="BF12" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="BG12" s="124"/>
-      <c r="BH12" s="124"/>
-      <c r="BI12" s="124" t="s">
+      <c r="BG12" s="191"/>
+      <c r="BH12" s="191"/>
+      <c r="BI12" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="BJ12" s="124"/>
-      <c r="BK12" s="124"/>
-      <c r="BL12" s="124" t="s">
+      <c r="BJ12" s="191"/>
+      <c r="BK12" s="191"/>
+      <c r="BL12" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="BM12" s="124"/>
-      <c r="BN12" s="124"/>
-      <c r="BO12" s="124" t="s">
+      <c r="BM12" s="191"/>
+      <c r="BN12" s="191"/>
+      <c r="BO12" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="BP12" s="124"/>
-      <c r="BQ12" s="176"/>
+      <c r="BP12" s="191"/>
+      <c r="BQ12" s="193"/>
       <c r="BS12" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="BT12" s="124" t="s">
+      <c r="BT12" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="BU12" s="124"/>
-      <c r="BV12" s="124"/>
-      <c r="BW12" s="124" t="s">
+      <c r="BU12" s="191"/>
+      <c r="BV12" s="191"/>
+      <c r="BW12" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="BX12" s="124"/>
-      <c r="BY12" s="124"/>
-      <c r="BZ12" s="124" t="s">
+      <c r="BX12" s="191"/>
+      <c r="BY12" s="191"/>
+      <c r="BZ12" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="CA12" s="124"/>
-      <c r="CB12" s="124"/>
-      <c r="CC12" s="124" t="s">
+      <c r="CA12" s="191"/>
+      <c r="CB12" s="191"/>
+      <c r="CC12" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="CD12" s="124"/>
-      <c r="CE12" s="124"/>
-      <c r="CF12" s="124" t="s">
+      <c r="CD12" s="191"/>
+      <c r="CE12" s="191"/>
+      <c r="CF12" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="CG12" s="124"/>
-      <c r="CH12" s="124"/>
-      <c r="CI12" s="124" t="s">
+      <c r="CG12" s="191"/>
+      <c r="CH12" s="191"/>
+      <c r="CI12" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="CJ12" s="124"/>
-      <c r="CK12" s="124"/>
-      <c r="CL12" s="124" t="s">
+      <c r="CJ12" s="191"/>
+      <c r="CK12" s="191"/>
+      <c r="CL12" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="CM12" s="124"/>
-      <c r="CN12" s="176"/>
+      <c r="CM12" s="191"/>
+      <c r="CN12" s="193"/>
     </row>
     <row r="13" spans="2:92" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="165">
@@ -8819,155 +8829,155 @@
       <c r="B28" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="124" t="s">
+      <c r="C28" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="D28" s="124"/>
-      <c r="E28" s="124"/>
-      <c r="F28" s="124" t="s">
+      <c r="D28" s="191"/>
+      <c r="E28" s="191"/>
+      <c r="F28" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="G28" s="124"/>
-      <c r="H28" s="124"/>
-      <c r="I28" s="124" t="s">
+      <c r="G28" s="191"/>
+      <c r="H28" s="191"/>
+      <c r="I28" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="J28" s="124"/>
-      <c r="K28" s="124"/>
-      <c r="L28" s="124" t="s">
+      <c r="J28" s="191"/>
+      <c r="K28" s="191"/>
+      <c r="L28" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="M28" s="124"/>
-      <c r="N28" s="124"/>
-      <c r="O28" s="124" t="s">
+      <c r="M28" s="191"/>
+      <c r="N28" s="191"/>
+      <c r="O28" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="P28" s="124"/>
-      <c r="Q28" s="124"/>
-      <c r="R28" s="124" t="s">
+      <c r="P28" s="191"/>
+      <c r="Q28" s="191"/>
+      <c r="R28" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="S28" s="124"/>
-      <c r="T28" s="124"/>
-      <c r="U28" s="124" t="s">
+      <c r="S28" s="191"/>
+      <c r="T28" s="191"/>
+      <c r="U28" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="V28" s="124"/>
-      <c r="W28" s="176"/>
+      <c r="V28" s="191"/>
+      <c r="W28" s="193"/>
       <c r="Y28" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="Z28" s="124" t="s">
+      <c r="Z28" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="AA28" s="124"/>
-      <c r="AB28" s="124"/>
-      <c r="AC28" s="124" t="s">
+      <c r="AA28" s="191"/>
+      <c r="AB28" s="191"/>
+      <c r="AC28" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="AD28" s="124"/>
-      <c r="AE28" s="124"/>
-      <c r="AF28" s="124" t="s">
+      <c r="AD28" s="191"/>
+      <c r="AE28" s="191"/>
+      <c r="AF28" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="AG28" s="124"/>
-      <c r="AH28" s="124"/>
-      <c r="AI28" s="124" t="s">
+      <c r="AG28" s="191"/>
+      <c r="AH28" s="191"/>
+      <c r="AI28" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="AJ28" s="124"/>
-      <c r="AK28" s="124"/>
-      <c r="AL28" s="124" t="s">
+      <c r="AJ28" s="191"/>
+      <c r="AK28" s="191"/>
+      <c r="AL28" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="AM28" s="124"/>
-      <c r="AN28" s="124"/>
-      <c r="AO28" s="124" t="s">
+      <c r="AM28" s="191"/>
+      <c r="AN28" s="191"/>
+      <c r="AO28" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="AP28" s="124"/>
-      <c r="AQ28" s="124"/>
-      <c r="AR28" s="124" t="s">
+      <c r="AP28" s="191"/>
+      <c r="AQ28" s="191"/>
+      <c r="AR28" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="AS28" s="124"/>
-      <c r="AT28" s="176"/>
+      <c r="AS28" s="191"/>
+      <c r="AT28" s="193"/>
       <c r="AV28" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="AW28" s="124" t="s">
+      <c r="AW28" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="AX28" s="124"/>
-      <c r="AY28" s="124"/>
-      <c r="AZ28" s="124" t="s">
+      <c r="AX28" s="191"/>
+      <c r="AY28" s="191"/>
+      <c r="AZ28" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="BA28" s="124"/>
-      <c r="BB28" s="124"/>
-      <c r="BC28" s="124" t="s">
+      <c r="BA28" s="191"/>
+      <c r="BB28" s="191"/>
+      <c r="BC28" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="BD28" s="124"/>
-      <c r="BE28" s="124"/>
-      <c r="BF28" s="124" t="s">
+      <c r="BD28" s="191"/>
+      <c r="BE28" s="191"/>
+      <c r="BF28" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="BG28" s="124"/>
-      <c r="BH28" s="124"/>
-      <c r="BI28" s="124" t="s">
+      <c r="BG28" s="191"/>
+      <c r="BH28" s="191"/>
+      <c r="BI28" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="BJ28" s="124"/>
-      <c r="BK28" s="124"/>
-      <c r="BL28" s="124" t="s">
+      <c r="BJ28" s="191"/>
+      <c r="BK28" s="191"/>
+      <c r="BL28" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="BM28" s="124"/>
-      <c r="BN28" s="124"/>
-      <c r="BO28" s="124" t="s">
+      <c r="BM28" s="191"/>
+      <c r="BN28" s="191"/>
+      <c r="BO28" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="BP28" s="124"/>
-      <c r="BQ28" s="176"/>
+      <c r="BP28" s="191"/>
+      <c r="BQ28" s="193"/>
       <c r="BS28" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="BT28" s="124" t="s">
+      <c r="BT28" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="BU28" s="124"/>
-      <c r="BV28" s="124"/>
-      <c r="BW28" s="124" t="s">
+      <c r="BU28" s="191"/>
+      <c r="BV28" s="191"/>
+      <c r="BW28" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="BX28" s="124"/>
-      <c r="BY28" s="124"/>
-      <c r="BZ28" s="124" t="s">
+      <c r="BX28" s="191"/>
+      <c r="BY28" s="191"/>
+      <c r="BZ28" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="CA28" s="124"/>
-      <c r="CB28" s="124"/>
-      <c r="CC28" s="124" t="s">
+      <c r="CA28" s="191"/>
+      <c r="CB28" s="191"/>
+      <c r="CC28" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="CD28" s="124"/>
-      <c r="CE28" s="124"/>
-      <c r="CF28" s="124" t="s">
+      <c r="CD28" s="191"/>
+      <c r="CE28" s="191"/>
+      <c r="CF28" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="CG28" s="124"/>
-      <c r="CH28" s="124"/>
-      <c r="CI28" s="124" t="s">
+      <c r="CG28" s="191"/>
+      <c r="CH28" s="191"/>
+      <c r="CI28" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="CJ28" s="124"/>
-      <c r="CK28" s="124"/>
-      <c r="CL28" s="124" t="s">
+      <c r="CJ28" s="191"/>
+      <c r="CK28" s="191"/>
+      <c r="CL28" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="CM28" s="124"/>
-      <c r="CN28" s="176"/>
+      <c r="CM28" s="191"/>
+      <c r="CN28" s="193"/>
     </row>
     <row r="29" spans="2:92" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="177">
@@ -12346,155 +12356,155 @@
       <c r="B44" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="124" t="s">
+      <c r="C44" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="D44" s="124"/>
-      <c r="E44" s="124"/>
-      <c r="F44" s="124" t="s">
+      <c r="D44" s="191"/>
+      <c r="E44" s="191"/>
+      <c r="F44" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="G44" s="124"/>
-      <c r="H44" s="124"/>
-      <c r="I44" s="124" t="s">
+      <c r="G44" s="191"/>
+      <c r="H44" s="191"/>
+      <c r="I44" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="J44" s="124"/>
-      <c r="K44" s="124"/>
-      <c r="L44" s="124" t="s">
+      <c r="J44" s="191"/>
+      <c r="K44" s="191"/>
+      <c r="L44" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="M44" s="124"/>
-      <c r="N44" s="124"/>
-      <c r="O44" s="124" t="s">
+      <c r="M44" s="191"/>
+      <c r="N44" s="191"/>
+      <c r="O44" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="P44" s="124"/>
-      <c r="Q44" s="124"/>
-      <c r="R44" s="124" t="s">
+      <c r="P44" s="191"/>
+      <c r="Q44" s="191"/>
+      <c r="R44" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="S44" s="124"/>
-      <c r="T44" s="124"/>
-      <c r="U44" s="124" t="s">
+      <c r="S44" s="191"/>
+      <c r="T44" s="191"/>
+      <c r="U44" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="V44" s="124"/>
-      <c r="W44" s="176"/>
+      <c r="V44" s="191"/>
+      <c r="W44" s="193"/>
       <c r="Y44" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="Z44" s="124" t="s">
+      <c r="Z44" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="AA44" s="124"/>
-      <c r="AB44" s="124"/>
-      <c r="AC44" s="124" t="s">
+      <c r="AA44" s="191"/>
+      <c r="AB44" s="191"/>
+      <c r="AC44" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="AD44" s="124"/>
-      <c r="AE44" s="124"/>
-      <c r="AF44" s="124" t="s">
+      <c r="AD44" s="191"/>
+      <c r="AE44" s="191"/>
+      <c r="AF44" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="AG44" s="124"/>
-      <c r="AH44" s="124"/>
-      <c r="AI44" s="124" t="s">
+      <c r="AG44" s="191"/>
+      <c r="AH44" s="191"/>
+      <c r="AI44" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="AJ44" s="124"/>
-      <c r="AK44" s="124"/>
-      <c r="AL44" s="124" t="s">
+      <c r="AJ44" s="191"/>
+      <c r="AK44" s="191"/>
+      <c r="AL44" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="AM44" s="124"/>
-      <c r="AN44" s="124"/>
-      <c r="AO44" s="124" t="s">
+      <c r="AM44" s="191"/>
+      <c r="AN44" s="191"/>
+      <c r="AO44" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="AP44" s="124"/>
-      <c r="AQ44" s="124"/>
-      <c r="AR44" s="124" t="s">
+      <c r="AP44" s="191"/>
+      <c r="AQ44" s="191"/>
+      <c r="AR44" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="AS44" s="124"/>
-      <c r="AT44" s="176"/>
+      <c r="AS44" s="191"/>
+      <c r="AT44" s="193"/>
       <c r="AV44" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="AW44" s="124" t="s">
+      <c r="AW44" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="AX44" s="124"/>
-      <c r="AY44" s="124"/>
-      <c r="AZ44" s="124" t="s">
+      <c r="AX44" s="191"/>
+      <c r="AY44" s="191"/>
+      <c r="AZ44" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="BA44" s="124"/>
-      <c r="BB44" s="124"/>
-      <c r="BC44" s="124" t="s">
+      <c r="BA44" s="191"/>
+      <c r="BB44" s="191"/>
+      <c r="BC44" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="BD44" s="124"/>
-      <c r="BE44" s="124"/>
-      <c r="BF44" s="124" t="s">
+      <c r="BD44" s="191"/>
+      <c r="BE44" s="191"/>
+      <c r="BF44" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="BG44" s="124"/>
-      <c r="BH44" s="124"/>
-      <c r="BI44" s="124" t="s">
+      <c r="BG44" s="191"/>
+      <c r="BH44" s="191"/>
+      <c r="BI44" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="BJ44" s="124"/>
-      <c r="BK44" s="124"/>
-      <c r="BL44" s="124" t="s">
+      <c r="BJ44" s="191"/>
+      <c r="BK44" s="191"/>
+      <c r="BL44" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="BM44" s="124"/>
-      <c r="BN44" s="124"/>
-      <c r="BO44" s="124" t="s">
+      <c r="BM44" s="191"/>
+      <c r="BN44" s="191"/>
+      <c r="BO44" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="BP44" s="124"/>
-      <c r="BQ44" s="176"/>
+      <c r="BP44" s="191"/>
+      <c r="BQ44" s="193"/>
       <c r="BS44" s="175" t="s">
         <v>72</v>
       </c>
-      <c r="BT44" s="124" t="s">
+      <c r="BT44" s="191" t="s">
         <v>73</v>
       </c>
-      <c r="BU44" s="124"/>
-      <c r="BV44" s="124"/>
-      <c r="BW44" s="124" t="s">
+      <c r="BU44" s="191"/>
+      <c r="BV44" s="191"/>
+      <c r="BW44" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="BX44" s="124"/>
-      <c r="BY44" s="124"/>
-      <c r="BZ44" s="124" t="s">
+      <c r="BX44" s="191"/>
+      <c r="BY44" s="191"/>
+      <c r="BZ44" s="191" t="s">
         <v>75</v>
       </c>
-      <c r="CA44" s="124"/>
-      <c r="CB44" s="124"/>
-      <c r="CC44" s="124" t="s">
+      <c r="CA44" s="191"/>
+      <c r="CB44" s="191"/>
+      <c r="CC44" s="191" t="s">
         <v>76</v>
       </c>
-      <c r="CD44" s="124"/>
-      <c r="CE44" s="124"/>
-      <c r="CF44" s="124" t="s">
+      <c r="CD44" s="191"/>
+      <c r="CE44" s="191"/>
+      <c r="CF44" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="CG44" s="124"/>
-      <c r="CH44" s="124"/>
-      <c r="CI44" s="124" t="s">
+      <c r="CG44" s="191"/>
+      <c r="CH44" s="191"/>
+      <c r="CI44" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="CJ44" s="124"/>
-      <c r="CK44" s="124"/>
-      <c r="CL44" s="124" t="s">
+      <c r="CJ44" s="191"/>
+      <c r="CK44" s="191"/>
+      <c r="CL44" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="CM44" s="124"/>
-      <c r="CN44" s="176"/>
+      <c r="CM44" s="191"/>
+      <c r="CN44" s="193"/>
     </row>
     <row r="45" spans="2:92" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="177">
@@ -16017,7 +16027,6 @@
       <c r="AG62" s="186"/>
       <c r="AH62" s="187"/>
       <c r="AI62" s="137">
-        <f t="shared" ref="AI62:AI81" si="1">IF($B62="","",Std_Vorlauf_Sel)</f>
         <v>76</v>
       </c>
       <c r="AJ62" s="137"/>
@@ -16037,7 +16046,6 @@
       <c r="AU62" s="136"/>
       <c r="AV62" s="136"/>
       <c r="AW62" s="137">
-        <f t="shared" ref="AW62:AW81" si="3">IF($B62="","",Std_Vorlauf_Inhalt)</f>
         <v>58</v>
       </c>
       <c r="AX62" s="137"/>
@@ -16237,7 +16245,6 @@
       <c r="AG64" s="136"/>
       <c r="AH64" s="136"/>
       <c r="AI64" s="137">
-        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="AJ64" s="137"/>
@@ -16257,7 +16264,6 @@
       <c r="AU64" s="136"/>
       <c r="AV64" s="136"/>
       <c r="AW64" s="137">
-        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="AX64" s="137"/>
@@ -16347,8 +16353,8 @@
       <c r="AF65" s="136"/>
       <c r="AG65" s="136"/>
       <c r="AH65" s="136"/>
-      <c r="AI65" s="137">
-        <f t="shared" si="1"/>
+      <c r="AI65" s="194">
+        <f>IF($BD65="","",Sommermailing!$C$4-Sommermailing!$F$11)</f>
         <v>76</v>
       </c>
       <c r="AJ65" s="137"/>
@@ -16367,8 +16373,8 @@
       <c r="AT65" s="136"/>
       <c r="AU65" s="136"/>
       <c r="AV65" s="136"/>
-      <c r="AW65" s="137">
-        <f t="shared" si="3"/>
+      <c r="AW65" s="195">
+        <f>IF($BD65="","",Sommermailing!$C$4-Sommermailing!$F$17)</f>
         <v>58</v>
       </c>
       <c r="AX65" s="137"/>
@@ -16461,7 +16467,6 @@
       <c r="AG66" s="136"/>
       <c r="AH66" s="136"/>
       <c r="AI66" s="137">
-        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="AJ66" s="137"/>
@@ -16481,7 +16486,6 @@
       <c r="AU66" s="136"/>
       <c r="AV66" s="136"/>
       <c r="AW66" s="137">
-        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="AX66" s="137"/>
@@ -16572,7 +16576,6 @@
       <c r="AG67" s="136"/>
       <c r="AH67" s="136"/>
       <c r="AI67" s="137">
-        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="AJ67" s="137"/>
@@ -16592,7 +16595,6 @@
       <c r="AU67" s="136"/>
       <c r="AV67" s="136"/>
       <c r="AW67" s="137">
-        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="AX67" s="137"/>
@@ -16683,7 +16685,6 @@
       <c r="AG68" s="136"/>
       <c r="AH68" s="136"/>
       <c r="AI68" s="137">
-        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="AJ68" s="137"/>
@@ -16703,7 +16704,6 @@
       <c r="AU68" s="136"/>
       <c r="AV68" s="136"/>
       <c r="AW68" s="137">
-        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="AX68" s="137"/>
@@ -16796,7 +16796,6 @@
       <c r="AG69" s="136"/>
       <c r="AH69" s="136"/>
       <c r="AI69" s="137">
-        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="AJ69" s="137"/>
@@ -16816,7 +16815,6 @@
       <c r="AU69" s="136"/>
       <c r="AV69" s="136"/>
       <c r="AW69" s="137">
-        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="AX69" s="137"/>
@@ -16906,8 +16904,8 @@
       <c r="AF70" s="136"/>
       <c r="AG70" s="136"/>
       <c r="AH70" s="136"/>
-      <c r="AI70" s="137">
-        <f t="shared" si="1"/>
+      <c r="AI70" s="196">
+        <f>IF($BD70="","",Weihnachtsmailing!$C$4-Weihnachtsmailing!$F$11)</f>
         <v>76</v>
       </c>
       <c r="AJ70" s="137"/>
@@ -16926,8 +16924,8 @@
       <c r="AT70" s="136"/>
       <c r="AU70" s="136"/>
       <c r="AV70" s="136"/>
-      <c r="AW70" s="137">
-        <f t="shared" si="3"/>
+      <c r="AW70" s="197">
+        <f>IF($BD70="","",Weihnachtsmailing!$C$4-Weihnachtsmailing!$F$17)</f>
         <v>58</v>
       </c>
       <c r="AX70" s="137"/>
@@ -17020,7 +17018,6 @@
       <c r="AG71" s="136"/>
       <c r="AH71" s="136"/>
       <c r="AI71" s="137">
-        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="AJ71" s="137"/>
@@ -17040,7 +17037,6 @@
       <c r="AU71" s="136"/>
       <c r="AV71" s="136"/>
       <c r="AW71" s="137">
-        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="AX71" s="137"/>
@@ -17128,10 +17124,7 @@
       <c r="AF72" s="136"/>
       <c r="AG72" s="136"/>
       <c r="AH72" s="136"/>
-      <c r="AI72" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI72" s="137"/>
       <c r="AJ72" s="137"/>
       <c r="AK72" s="137"/>
       <c r="AL72" s="137"/>
@@ -17148,10 +17141,7 @@
       <c r="AT72" s="136"/>
       <c r="AU72" s="136"/>
       <c r="AV72" s="136"/>
-      <c r="AW72" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW72" s="137"/>
       <c r="AX72" s="137"/>
       <c r="AY72" s="137"/>
       <c r="AZ72" s="137"/>
@@ -17233,10 +17223,7 @@
       <c r="AF73" s="136"/>
       <c r="AG73" s="136"/>
       <c r="AH73" s="136"/>
-      <c r="AI73" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI73" s="137"/>
       <c r="AJ73" s="137"/>
       <c r="AK73" s="137"/>
       <c r="AL73" s="137"/>
@@ -17253,10 +17240,7 @@
       <c r="AT73" s="136"/>
       <c r="AU73" s="136"/>
       <c r="AV73" s="136"/>
-      <c r="AW73" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW73" s="137"/>
       <c r="AX73" s="137"/>
       <c r="AY73" s="137"/>
       <c r="AZ73" s="137"/>
@@ -17338,10 +17322,7 @@
       <c r="AF74" s="136"/>
       <c r="AG74" s="136"/>
       <c r="AH74" s="136"/>
-      <c r="AI74" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI74" s="137"/>
       <c r="AJ74" s="137"/>
       <c r="AK74" s="137"/>
       <c r="AL74" s="137"/>
@@ -17358,10 +17339,7 @@
       <c r="AT74" s="136"/>
       <c r="AU74" s="136"/>
       <c r="AV74" s="136"/>
-      <c r="AW74" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW74" s="137"/>
       <c r="AX74" s="137"/>
       <c r="AY74" s="137"/>
       <c r="AZ74" s="137"/>
@@ -17443,10 +17421,7 @@
       <c r="AF75" s="136"/>
       <c r="AG75" s="136"/>
       <c r="AH75" s="136"/>
-      <c r="AI75" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI75" s="137"/>
       <c r="AJ75" s="137"/>
       <c r="AK75" s="137"/>
       <c r="AL75" s="137"/>
@@ -17463,10 +17438,7 @@
       <c r="AT75" s="136"/>
       <c r="AU75" s="136"/>
       <c r="AV75" s="136"/>
-      <c r="AW75" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW75" s="137"/>
       <c r="AX75" s="137"/>
       <c r="AY75" s="137"/>
       <c r="AZ75" s="137"/>
@@ -17548,10 +17520,7 @@
       <c r="AF76" s="136"/>
       <c r="AG76" s="136"/>
       <c r="AH76" s="136"/>
-      <c r="AI76" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI76" s="137"/>
       <c r="AJ76" s="137"/>
       <c r="AK76" s="137"/>
       <c r="AL76" s="137"/>
@@ -17568,10 +17537,7 @@
       <c r="AT76" s="136"/>
       <c r="AU76" s="136"/>
       <c r="AV76" s="136"/>
-      <c r="AW76" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW76" s="137"/>
       <c r="AX76" s="137"/>
       <c r="AY76" s="137"/>
       <c r="AZ76" s="137"/>
@@ -17653,10 +17619,7 @@
       <c r="AF77" s="136"/>
       <c r="AG77" s="136"/>
       <c r="AH77" s="136"/>
-      <c r="AI77" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI77" s="137"/>
       <c r="AJ77" s="137"/>
       <c r="AK77" s="137"/>
       <c r="AL77" s="137"/>
@@ -17673,10 +17636,7 @@
       <c r="AT77" s="136"/>
       <c r="AU77" s="136"/>
       <c r="AV77" s="136"/>
-      <c r="AW77" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW77" s="137"/>
       <c r="AX77" s="137"/>
       <c r="AY77" s="137"/>
       <c r="AZ77" s="137"/>
@@ -17758,10 +17718,7 @@
       <c r="AF78" s="136"/>
       <c r="AG78" s="136"/>
       <c r="AH78" s="136"/>
-      <c r="AI78" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI78" s="137"/>
       <c r="AJ78" s="137"/>
       <c r="AK78" s="137"/>
       <c r="AL78" s="137"/>
@@ -17778,10 +17735,7 @@
       <c r="AT78" s="136"/>
       <c r="AU78" s="136"/>
       <c r="AV78" s="136"/>
-      <c r="AW78" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW78" s="137"/>
       <c r="AX78" s="137"/>
       <c r="AY78" s="137"/>
       <c r="AZ78" s="137"/>
@@ -17863,10 +17817,7 @@
       <c r="AF79" s="136"/>
       <c r="AG79" s="136"/>
       <c r="AH79" s="136"/>
-      <c r="AI79" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI79" s="137"/>
       <c r="AJ79" s="137"/>
       <c r="AK79" s="137"/>
       <c r="AL79" s="137"/>
@@ -17883,10 +17834,7 @@
       <c r="AT79" s="136"/>
       <c r="AU79" s="136"/>
       <c r="AV79" s="136"/>
-      <c r="AW79" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW79" s="137"/>
       <c r="AX79" s="137"/>
       <c r="AY79" s="137"/>
       <c r="AZ79" s="137"/>
@@ -17968,10 +17916,7 @@
       <c r="AF80" s="136"/>
       <c r="AG80" s="136"/>
       <c r="AH80" s="136"/>
-      <c r="AI80" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI80" s="137"/>
       <c r="AJ80" s="137"/>
       <c r="AK80" s="137"/>
       <c r="AL80" s="137"/>
@@ -17988,10 +17933,7 @@
       <c r="AT80" s="136"/>
       <c r="AU80" s="136"/>
       <c r="AV80" s="136"/>
-      <c r="AW80" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW80" s="137"/>
       <c r="AX80" s="137"/>
       <c r="AY80" s="137"/>
       <c r="AZ80" s="137"/>
@@ -18073,10 +18015,7 @@
       <c r="AF81" s="136"/>
       <c r="AG81" s="136"/>
       <c r="AH81" s="136"/>
-      <c r="AI81" s="137" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="AI81" s="137"/>
       <c r="AJ81" s="137"/>
       <c r="AK81" s="137"/>
       <c r="AL81" s="137"/>
@@ -18093,10 +18032,7 @@
       <c r="AT81" s="136"/>
       <c r="AU81" s="136"/>
       <c r="AV81" s="136"/>
-      <c r="AW81" s="137" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="AW81" s="137"/>
       <c r="AX81" s="137"/>
       <c r="AY81" s="137"/>
       <c r="AZ81" s="137"/>
@@ -18333,7 +18269,7 @@
     </row>
     <row r="85" spans="2:92" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="142" t="s">
-        <v>99</v>
+        <v>152</v>
       </c>
       <c r="C85" s="142"/>
       <c r="D85" s="142"/>
@@ -18428,7 +18364,7 @@
     </row>
     <row r="86" spans="2:92" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="142" t="s">
-        <v>100</v>
+        <v>153</v>
       </c>
       <c r="C86" s="142"/>
       <c r="D86" s="142"/>
@@ -18617,7 +18553,7 @@
       <c r="CN87" s="142"/>
     </row>
   </sheetData>
-  <mergeCells count="829">
+  <mergeCells count="739">
     <mergeCell ref="B83:CN83"/>
     <mergeCell ref="B84:CN84"/>
     <mergeCell ref="B85:CN85"/>
@@ -18844,13 +18780,6 @@
     <mergeCell ref="CL51:CN51"/>
     <mergeCell ref="AV57:BQ57"/>
     <mergeCell ref="BS43:CN43"/>
-    <mergeCell ref="BT44:BV44"/>
-    <mergeCell ref="BW44:BY44"/>
-    <mergeCell ref="BZ44:CB44"/>
-    <mergeCell ref="CC44:CE44"/>
-    <mergeCell ref="CF44:CH44"/>
-    <mergeCell ref="CI44:CK44"/>
-    <mergeCell ref="CL44:CN44"/>
     <mergeCell ref="BT45:BV45"/>
     <mergeCell ref="BW45:BY45"/>
     <mergeCell ref="BZ45:CB45"/>
@@ -18895,13 +18824,6 @@
     <mergeCell ref="BO51:BQ51"/>
     <mergeCell ref="Y57:AT57"/>
     <mergeCell ref="AV43:BQ43"/>
-    <mergeCell ref="AW44:AY44"/>
-    <mergeCell ref="AZ44:BB44"/>
-    <mergeCell ref="BC44:BE44"/>
-    <mergeCell ref="BF44:BH44"/>
-    <mergeCell ref="BI44:BK44"/>
-    <mergeCell ref="BL44:BN44"/>
-    <mergeCell ref="BO44:BQ44"/>
     <mergeCell ref="AW45:AY45"/>
     <mergeCell ref="AZ45:BB45"/>
     <mergeCell ref="BC45:BE45"/>
@@ -18946,13 +18868,6 @@
     <mergeCell ref="AR51:AT51"/>
     <mergeCell ref="B57:W57"/>
     <mergeCell ref="Y43:AT43"/>
-    <mergeCell ref="Z44:AB44"/>
-    <mergeCell ref="AC44:AE44"/>
-    <mergeCell ref="AF44:AH44"/>
-    <mergeCell ref="AI44:AK44"/>
-    <mergeCell ref="AL44:AN44"/>
-    <mergeCell ref="AO44:AQ44"/>
-    <mergeCell ref="AR44:AT44"/>
     <mergeCell ref="Z45:AB45"/>
     <mergeCell ref="AC45:AE45"/>
     <mergeCell ref="AF45:AH45"/>
@@ -19012,13 +18927,6 @@
     <mergeCell ref="U47:W47"/>
     <mergeCell ref="BS41:CN41"/>
     <mergeCell ref="B43:W43"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="F44:H44"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="O44:Q44"/>
-    <mergeCell ref="R44:T44"/>
-    <mergeCell ref="U44:W44"/>
     <mergeCell ref="BT37:BV37"/>
     <mergeCell ref="BW37:BY37"/>
     <mergeCell ref="BZ37:CB37"/>
@@ -19048,13 +18956,6 @@
     <mergeCell ref="CL35:CN35"/>
     <mergeCell ref="AV41:BQ41"/>
     <mergeCell ref="BS27:CN27"/>
-    <mergeCell ref="BT28:BV28"/>
-    <mergeCell ref="BW28:BY28"/>
-    <mergeCell ref="BZ28:CB28"/>
-    <mergeCell ref="CC28:CE28"/>
-    <mergeCell ref="CF28:CH28"/>
-    <mergeCell ref="CI28:CK28"/>
-    <mergeCell ref="CL28:CN28"/>
     <mergeCell ref="BT29:BV29"/>
     <mergeCell ref="BW29:BY29"/>
     <mergeCell ref="BZ29:CB29"/>
@@ -19099,13 +19000,6 @@
     <mergeCell ref="BO35:BQ35"/>
     <mergeCell ref="Y41:AT41"/>
     <mergeCell ref="AV27:BQ27"/>
-    <mergeCell ref="AW28:AY28"/>
-    <mergeCell ref="AZ28:BB28"/>
-    <mergeCell ref="BC28:BE28"/>
-    <mergeCell ref="BF28:BH28"/>
-    <mergeCell ref="BI28:BK28"/>
-    <mergeCell ref="BL28:BN28"/>
-    <mergeCell ref="BO28:BQ28"/>
     <mergeCell ref="AW29:AY29"/>
     <mergeCell ref="AZ29:BB29"/>
     <mergeCell ref="BC29:BE29"/>
@@ -19150,13 +19044,6 @@
     <mergeCell ref="AR35:AT35"/>
     <mergeCell ref="B41:W41"/>
     <mergeCell ref="Y27:AT27"/>
-    <mergeCell ref="Z28:AB28"/>
-    <mergeCell ref="AC28:AE28"/>
-    <mergeCell ref="AF28:AH28"/>
-    <mergeCell ref="AI28:AK28"/>
-    <mergeCell ref="AL28:AN28"/>
-    <mergeCell ref="AO28:AQ28"/>
-    <mergeCell ref="AR28:AT28"/>
     <mergeCell ref="Z29:AB29"/>
     <mergeCell ref="AC29:AE29"/>
     <mergeCell ref="AF29:AH29"/>
@@ -19216,13 +19103,6 @@
     <mergeCell ref="U31:W31"/>
     <mergeCell ref="BS25:CN25"/>
     <mergeCell ref="B27:W27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="L28:N28"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="R28:T28"/>
-    <mergeCell ref="U28:W28"/>
     <mergeCell ref="BT21:BV21"/>
     <mergeCell ref="BW21:BY21"/>
     <mergeCell ref="BZ21:CB21"/>
@@ -19252,13 +19132,6 @@
     <mergeCell ref="CL19:CN19"/>
     <mergeCell ref="AV25:BQ25"/>
     <mergeCell ref="BS11:CN11"/>
-    <mergeCell ref="BT12:BV12"/>
-    <mergeCell ref="BW12:BY12"/>
-    <mergeCell ref="BZ12:CB12"/>
-    <mergeCell ref="CC12:CE12"/>
-    <mergeCell ref="CF12:CH12"/>
-    <mergeCell ref="CI12:CK12"/>
-    <mergeCell ref="CL12:CN12"/>
     <mergeCell ref="BT13:BV13"/>
     <mergeCell ref="BW13:BY13"/>
     <mergeCell ref="BZ13:CB13"/>
@@ -19303,13 +19176,6 @@
     <mergeCell ref="BO19:BQ19"/>
     <mergeCell ref="Y25:AT25"/>
     <mergeCell ref="AV11:BQ11"/>
-    <mergeCell ref="AW12:AY12"/>
-    <mergeCell ref="AZ12:BB12"/>
-    <mergeCell ref="BC12:BE12"/>
-    <mergeCell ref="BF12:BH12"/>
-    <mergeCell ref="BI12:BK12"/>
-    <mergeCell ref="BL12:BN12"/>
-    <mergeCell ref="BO12:BQ12"/>
     <mergeCell ref="AW13:AY13"/>
     <mergeCell ref="AZ13:BB13"/>
     <mergeCell ref="BC13:BE13"/>
@@ -19354,13 +19220,6 @@
     <mergeCell ref="AR19:AT19"/>
     <mergeCell ref="B25:W25"/>
     <mergeCell ref="Y11:AT11"/>
-    <mergeCell ref="Z12:AB12"/>
-    <mergeCell ref="AC12:AE12"/>
-    <mergeCell ref="AF12:AH12"/>
-    <mergeCell ref="AI12:AK12"/>
-    <mergeCell ref="AL12:AN12"/>
-    <mergeCell ref="AO12:AQ12"/>
-    <mergeCell ref="AR12:AT12"/>
     <mergeCell ref="Z13:AB13"/>
     <mergeCell ref="AC13:AE13"/>
     <mergeCell ref="AF13:AH13"/>
@@ -19420,26 +19279,13 @@
     <mergeCell ref="U15:W15"/>
     <mergeCell ref="B9:CN9"/>
     <mergeCell ref="B11:W11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="F12:H12"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="L12:N12"/>
-    <mergeCell ref="O12:Q12"/>
-    <mergeCell ref="R12:T12"/>
-    <mergeCell ref="U12:W12"/>
     <mergeCell ref="Q2:CN2"/>
     <mergeCell ref="B4:V4"/>
     <mergeCell ref="W4:AA4"/>
-    <mergeCell ref="B5:V5"/>
-    <mergeCell ref="W5:AA5"/>
-    <mergeCell ref="B6:V6"/>
-    <mergeCell ref="W6:AA6"/>
     <mergeCell ref="B7:AC7"/>
     <mergeCell ref="AE4:BQ4"/>
     <mergeCell ref="AE5:BQ5"/>
     <mergeCell ref="AE6:BQ6"/>
-    <mergeCell ref="AE7:AV7"/>
-    <mergeCell ref="AX7:BQ7"/>
     <mergeCell ref="BV4:CN4"/>
     <mergeCell ref="BV5:CN5"/>
     <mergeCell ref="BV6:CN6"/>
@@ -19449,517 +19295,632 @@
     <mergeCell ref="CF7:CN7"/>
   </mergeCells>
   <conditionalFormatting sqref="C13 F13 I13 L13 O13 R13 U13 C15 F15 I15 L15 O15 R15 U15 C17 F17 I17 L17 O17 R17 U17 C19 F19 I19 L19 O19 R19 U19 C21 F21 I21 L21 O21 R21 U21 C23 F23 I23 L23 O23 R23 U23">
-    <cfRule type="expression" dxfId="130" priority="1">
+    <cfRule type="expression" dxfId="136" priority="1">
       <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D13 G13 J13 M13 P13 S13 V13 D15 G15 J15 M15 P15 S15 V15 D17 G17 J17 M17 P17 S17 V17 D19 G19 J19 M19 P19 S19 V19 D21 G21 J21 M21 P21 S21 V21 D23 G23 J23 M23 P23 S23 V23">
-    <cfRule type="expression" dxfId="131" priority="2">
+  <conditionalFormatting sqref="C12 F12 I12 L12 O12 R12 U12 C14 F14 I14 L14 O14 R14 U14 C16 F16 I16 L16 O16 R16 U16 C18 F18 I18 L18 O18 R18 U18 C20 F20 I20 L20 O20 R20 U20 C22 F22 I22 L22 O22 R22 U22">
+    <cfRule type="expression" dxfId="137" priority="2">
       <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E13 H13 K13 N13 Q13 T13 W13 E15 H15 K15 N15 Q15 T15 W15 E17 H17 K17 N17 Q17 T17 W17 E19 H19 K19 N19 Q19 T19 W19 E21 H21 K21 N21 Q21 T21 W21 E23 H23 K23 N23 Q23 T23 W23">
-    <cfRule type="expression" dxfId="132" priority="3">
+  <conditionalFormatting sqref="D12 G12 J12 M12 P12 S12 V12 D14 G14 J14 M14 P14 S14 V14 D16 G16 J16 M16 P16 S16 V16 D18 G18 J18 M18 P18 S18 V18 D20 G20 J20 M20 P20 S20 V20 D22 G22 J22 M22 P22 S22 V22">
+    <cfRule type="expression" dxfId="137" priority="3">
+      <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12 H12 K12 N12 Q12 T12 W12 E14 H14 K14 N14 Q14 T14 W14 E16 H16 K16 N16 Q16 T16 W16 E18 H18 K18 N18 Q18 T18 W18 E20 H20 K20 N20 Q20 T20 W20 E22 H22 K22 N22 Q22 T22 W22">
+    <cfRule type="expression" dxfId="137" priority="4">
+      <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F13 I13 L13 O13 R13 U13 X13 F15 I15 L15 O15 R15 U15 X15 F17 I17 L17 O17 R17 U17 X17 F19 I19 L19 O19 R19 U19 X19 F21 I21 L21 O21 R21 U21 X21 F23 I23 L23 O23 R23 U23 X23">
+    <cfRule type="expression" dxfId="138" priority="5">
       <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14 F14 I14 L14 O14 R14 U14 C16 F16 I16 L16 O16 R16 U16 C18 F18 I18 L18 O18 R18 U18 C20 F20 I20 L20 O20 R20 U20 C22 F22 I22 L22 O22 R22 U22 C24 F24 I24 L24 O24 R24 U24">
-    <cfRule type="expression" dxfId="133" priority="4">
+    <cfRule type="expression" dxfId="139" priority="6">
       <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14 G14 J14 M14 P14 S14 V14 D16 G16 J16 M16 P16 S16 V16 D18 G18 J18 M18 P18 S18 V18 D20 G20 J20 M20 P20 S20 V20 D22 G22 J22 M22 P22 S22 V22 D24 G24 J24 M24 P24 S24 V24">
-    <cfRule type="expression" dxfId="134" priority="5">
+    <cfRule type="expression" dxfId="140" priority="7">
       <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14 H14 K14 N14 Q14 T14 W14 E16 H16 K16 N16 Q16 T16 W16 E18 H18 K18 N18 Q18 T18 W18 E20 H20 K20 N20 Q20 T20 W20 E22 H22 K22 N22 Q22 T22 W22 E24 H24 K24 N24 Q24 T24 W24">
-    <cfRule type="expression" dxfId="135" priority="6">
+    <cfRule type="expression" dxfId="141" priority="8">
       <formula>AND(ISNUMBER(C13),DATE(Planungsjahr,1,C13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z13 AC13 AF13 AI13 AL13 AO13 AR13 Z15 AC15 AF15 AI15 AL15 AO15 AR15 Z17 AC17 AF17 AI17 AL17 AO17 AR17 Z19 AC19 AF19 AI19 AL19 AO19 AR19 Z21 AC21 AF21 AI21 AL21 AO21 AR21 Z23 AC23 AF23 AI23 AL23 AO23 AR23">
-    <cfRule type="expression" dxfId="130" priority="7">
+    <cfRule type="expression" dxfId="136" priority="9">
       <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA13 AD13 AG13 AJ13 AM13 AP13 AS13 AA15 AD15 AG15 AJ15 AM15 AP15 AS15 AA17 AD17 AG17 AJ17 AM17 AP17 AS17 AA19 AD19 AG19 AJ19 AM19 AP19 AS19 AA21 AD21 AG21 AJ21 AM21 AP21 AS21 AA23 AD23 AG23 AJ23 AM23 AP23 AS23">
-    <cfRule type="expression" dxfId="131" priority="8">
+  <conditionalFormatting sqref="Z12 AC12 AF12 AI12 AL12 AO12 AR12 Z14 AC14 AF14 AI14 AL14 AO14 AR14 Z16 AC16 AF16 AI16 AL16 AO16 AR16 Z18 AC18 AF18 AI18 AL18 AO18 AR18 Z20 AC20 AF20 AI20 AL20 AO20 AR20 Z22 AC22 AF22 AI22 AL22 AO22 AR22">
+    <cfRule type="expression" dxfId="137" priority="10">
       <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB13 AE13 AH13 AK13 AN13 AQ13 AT13 AB15 AE15 AH15 AK15 AN15 AQ15 AT15 AB17 AE17 AH17 AK17 AN17 AQ17 AT17 AB19 AE19 AH19 AK19 AN19 AQ19 AT19 AB21 AE21 AH21 AK21 AN21 AQ21 AT21 AB23 AE23 AH23 AK23 AN23 AQ23 AT23">
-    <cfRule type="expression" dxfId="132" priority="9">
+  <conditionalFormatting sqref="AA12 AD12 AG12 AJ12 AM12 AP12 AS12 AA14 AD14 AG14 AJ14 AM14 AP14 AS14 AA16 AD16 AG16 AJ16 AM16 AP16 AS16 AA18 AD18 AG18 AJ18 AM18 AP18 AS18 AA20 AD20 AG20 AJ20 AM20 AP20 AS20 AA22 AD22 AG22 AJ22 AM22 AP22 AS22">
+    <cfRule type="expression" dxfId="137" priority="11">
+      <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB12 AE12 AH12 AK12 AN12 AQ12 AT12 AB14 AE14 AH14 AK14 AN14 AQ14 AT14 AB16 AE16 AH16 AK16 AN16 AQ16 AT16 AB18 AE18 AH18 AK18 AN18 AQ18 AT18 AB20 AE20 AH20 AK20 AN20 AQ20 AT20 AB22 AE22 AH22 AK22 AN22 AQ22 AT22">
+    <cfRule type="expression" dxfId="137" priority="12">
+      <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC13 AF13 AI13 AL13 AO13 AR13 AU13 AC15 AF15 AI15 AL15 AO15 AR15 AU15 AC17 AF17 AI17 AL17 AO17 AR17 AU17 AC19 AF19 AI19 AL19 AO19 AR19 AU19 AC21 AF21 AI21 AL21 AO21 AR21 AU21 AC23 AF23 AI23 AL23 AO23 AR23 AU23">
+    <cfRule type="expression" dxfId="138" priority="13">
       <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z14 AC14 AF14 AI14 AL14 AO14 AR14 Z16 AC16 AF16 AI16 AL16 AO16 AR16 Z18 AC18 AF18 AI18 AL18 AO18 AR18 Z20 AC20 AF20 AI20 AL20 AO20 AR20 Z22 AC22 AF22 AI22 AL22 AO22 AR22 Z24 AC24 AF24 AI24 AL24 AO24 AR24">
-    <cfRule type="expression" dxfId="133" priority="10">
+    <cfRule type="expression" dxfId="139" priority="14">
       <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA14 AD14 AG14 AJ14 AM14 AP14 AS14 AA16 AD16 AG16 AJ16 AM16 AP16 AS16 AA18 AD18 AG18 AJ18 AM18 AP18 AS18 AA20 AD20 AG20 AJ20 AM20 AP20 AS20 AA22 AD22 AG22 AJ22 AM22 AP22 AS22 AA24 AD24 AG24 AJ24 AM24 AP24 AS24">
-    <cfRule type="expression" dxfId="134" priority="11">
+    <cfRule type="expression" dxfId="140" priority="15">
       <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB14 AE14 AH14 AK14 AN14 AQ14 AT14 AB16 AE16 AH16 AK16 AN16 AQ16 AT16 AB18 AE18 AH18 AK18 AN18 AQ18 AT18 AB20 AE20 AH20 AK20 AN20 AQ20 AT20 AB22 AE22 AH22 AK22 AN22 AQ22 AT22 AB24 AE24 AH24 AK24 AN24 AQ24 AT24">
-    <cfRule type="expression" dxfId="135" priority="12">
+    <cfRule type="expression" dxfId="141" priority="16">
       <formula>AND(ISNUMBER(Z13),DATE(Planungsjahr,2,Z13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW13 AZ13 BC13 BF13 BI13 BL13 BO13 AW15 AZ15 BC15 BF15 BI15 BL15 BO15 AW17 AZ17 BC17 BF17 BI17 BL17 BO17 AW19 AZ19 BC19 BF19 BI19 BL19 BO19 AW21 AZ21 BC21 BF21 BI21 BL21 BO21 AW23 AZ23 BC23 BF23 BI23 BL23 BO23">
-    <cfRule type="expression" dxfId="130" priority="13">
+    <cfRule type="expression" dxfId="136" priority="17">
       <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AX13 BA13 BD13 BG13 BJ13 BM13 BP13 AX15 BA15 BD15 BG15 BJ15 BM15 BP15 AX17 BA17 BD17 BG17 BJ17 BM17 BP17 AX19 BA19 BD19 BG19 BJ19 BM19 BP19 AX21 BA21 BD21 BG21 BJ21 BM21 BP21 AX23 BA23 BD23 BG23 BJ23 BM23 BP23">
-    <cfRule type="expression" dxfId="131" priority="14">
+  <conditionalFormatting sqref="AW12 AZ12 BC12 BF12 BI12 BL12 BO12 AW14 AZ14 BC14 BF14 BI14 BL14 BO14 AW16 AZ16 BC16 BF16 BI16 BL16 BO16 AW18 AZ18 BC18 BF18 BI18 BL18 BO18 AW20 AZ20 BC20 BF20 BI20 BL20 BO20 AW22 AZ22 BC22 BF22 BI22 BL22 BO22">
+    <cfRule type="expression" dxfId="137" priority="18">
       <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AY13 BB13 BE13 BH13 BK13 BN13 BQ13 AY15 BB15 BE15 BH15 BK15 BN15 BQ15 AY17 BB17 BE17 BH17 BK17 BN17 BQ17 AY19 BB19 BE19 BH19 BK19 BN19 BQ19 AY21 BB21 BE21 BH21 BK21 BN21 BQ21 AY23 BB23 BE23 BH23 BK23 BN23 BQ23">
-    <cfRule type="expression" dxfId="132" priority="15">
+  <conditionalFormatting sqref="AX12 BA12 BD12 BG12 BJ12 BM12 BP12 AX14 BA14 BD14 BG14 BJ14 BM14 BP14 AX16 BA16 BD16 BG16 BJ16 BM16 BP16 AX18 BA18 BD18 BG18 BJ18 BM18 BP18 AX20 BA20 BD20 BG20 BJ20 BM20 BP20 AX22 BA22 BD22 BG22 BJ22 BM22 BP22">
+    <cfRule type="expression" dxfId="137" priority="19">
+      <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AY12 BB12 BE12 BH12 BK12 BN12 BQ12 AY14 BB14 BE14 BH14 BK14 BN14 BQ14 AY16 BB16 BE16 BH16 BK16 BN16 BQ16 AY18 BB18 BE18 BH18 BK18 BN18 BQ18 AY20 BB20 BE20 BH20 BK20 BN20 BQ20 AY22 BB22 BE22 BH22 BK22 BN22 BQ22">
+    <cfRule type="expression" dxfId="137" priority="20">
+      <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AZ13 BC13 BF13 BI13 BL13 BO13 BR13 AZ15 BC15 BF15 BI15 BL15 BO15 BR15 AZ17 BC17 BF17 BI17 BL17 BO17 BR17 AZ19 BC19 BF19 BI19 BL19 BO19 BR19 AZ21 BC21 BF21 BI21 BL21 BO21 BR21 AZ23 BC23 BF23 BI23 BL23 BO23 BR23">
+    <cfRule type="expression" dxfId="138" priority="21">
       <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW14 AZ14 BC14 BF14 BI14 BL14 BO14 AW16 AZ16 BC16 BF16 BI16 BL16 BO16 AW18 AZ18 BC18 BF18 BI18 BL18 BO18 AW20 AZ20 BC20 BF20 BI20 BL20 BO20 AW22 AZ22 BC22 BF22 BI22 BL22 BO22 AW24 AZ24 BC24 BF24 BI24 BL24 BO24">
-    <cfRule type="expression" dxfId="133" priority="16">
+    <cfRule type="expression" dxfId="139" priority="22">
       <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AX14 BA14 BD14 BG14 BJ14 BM14 BP14 AX16 BA16 BD16 BG16 BJ16 BM16 BP16 AX18 BA18 BD18 BG18 BJ18 BM18 BP18 AX20 BA20 BD20 BG20 BJ20 BM20 BP20 AX22 BA22 BD22 BG22 BJ22 BM22 BP22 AX24 BA24 BD24 BG24 BJ24 BM24 BP24">
-    <cfRule type="expression" dxfId="134" priority="17">
+    <cfRule type="expression" dxfId="140" priority="23">
       <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AY14 BB14 BE14 BH14 BK14 BN14 BQ14 AY16 BB16 BE16 BH16 BK16 BN16 BQ16 AY18 BB18 BE18 BH18 BK18 BN18 BQ18 AY20 BB20 BE20 BH20 BK20 BN20 BQ20 AY22 BB22 BE22 BH22 BK22 BN22 BQ22 AY24 BB24 BE24 BH24 BK24 BN24 BQ24">
-    <cfRule type="expression" dxfId="135" priority="18">
+    <cfRule type="expression" dxfId="141" priority="24">
       <formula>AND(ISNUMBER(AW13),DATE(Planungsjahr,3,AW13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT13 BW13 BZ13 CC13 CF13 CI13 CL13 BT15 BW15 BZ15 CC15 CF15 CI15 CL15 BT17 BW17 BZ17 CC17 CF17 CI17 CL17 BT19 BW19 BZ19 CC19 CF19 CI19 CL19 BT21 BW21 BZ21 CC21 CF21 CI21 CL21 BT23 BW23 BZ23 CC23 CF23 CI23 CL23">
-    <cfRule type="expression" dxfId="130" priority="19">
+    <cfRule type="expression" dxfId="136" priority="25">
       <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BU13 BX13 CA13 CD13 CG13 CJ13 CM13 BU15 BX15 CA15 CD15 CG15 CJ15 CM15 BU17 BX17 CA17 CD17 CG17 CJ17 CM17 BU19 BX19 CA19 CD19 CG19 CJ19 CM19 BU21 BX21 CA21 CD21 CG21 CJ21 CM21 BU23 BX23 CA23 CD23 CG23 CJ23 CM23">
-    <cfRule type="expression" dxfId="131" priority="20">
+  <conditionalFormatting sqref="BT12 BW12 BZ12 CC12 CF12 CI12 CL12 BT14 BW14 BZ14 CC14 CF14 CI14 CL14 BT16 BW16 BZ16 CC16 CF16 CI16 CL16 BT18 BW18 BZ18 CC18 CF18 CI18 CL18 BT20 BW20 BZ20 CC20 CF20 CI20 CL20 BT22 BW22 BZ22 CC22 CF22 CI22 CL22">
+    <cfRule type="expression" dxfId="137" priority="26">
       <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BV13 BY13 CB13 CE13 CH13 CK13 CN13 BV15 BY15 CB15 CE15 CH15 CK15 CN15 BV17 BY17 CB17 CE17 CH17 CK17 CN17 BV19 BY19 CB19 CE19 CH19 CK19 CN19 BV21 BY21 CB21 CE21 CH21 CK21 CN21 BV23 BY23 CB23 CE23 CH23 CK23 CN23">
-    <cfRule type="expression" dxfId="132" priority="21">
+  <conditionalFormatting sqref="BU12 BX12 CA12 CD12 CG12 CJ12 CM12 BU14 BX14 CA14 CD14 CG14 CJ14 CM14 BU16 BX16 CA16 CD16 CG16 CJ16 CM16 BU18 BX18 CA18 CD18 CG18 CJ18 CM18 BU20 BX20 CA20 CD20 CG20 CJ20 CM20 BU22 BX22 CA22 CD22 CG22 CJ22 CM22">
+    <cfRule type="expression" dxfId="137" priority="27">
+      <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BV12 BY12 CB12 CE12 CH12 CK12 CN12 BV14 BY14 CB14 CE14 CH14 CK14 CN14 BV16 BY16 CB16 CE16 CH16 CK16 CN16 BV18 BY18 CB18 CE18 CH18 CK18 CN18 BV20 BY20 CB20 CE20 CH20 CK20 CN20 BV22 BY22 CB22 CE22 CH22 CK22 CN22">
+    <cfRule type="expression" dxfId="137" priority="28">
+      <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BW13 BZ13 CC13 CF13 CI13 CL13 CO13 BW15 BZ15 CC15 CF15 CI15 CL15 CO15 BW17 BZ17 CC17 CF17 CI17 CL17 CO17 BW19 BZ19 CC19 CF19 CI19 CL19 CO19 BW21 BZ21 CC21 CF21 CI21 CL21 CO21 BW23 BZ23 CC23 CF23 CI23 CL23 CO23">
+    <cfRule type="expression" dxfId="138" priority="29">
       <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT14 BW14 BZ14 CC14 CF14 CI14 CL14 BT16 BW16 BZ16 CC16 CF16 CI16 CL16 BT18 BW18 BZ18 CC18 CF18 CI18 CL18 BT20 BW20 BZ20 CC20 CF20 CI20 CL20 BT22 BW22 BZ22 CC22 CF22 CI22 CL22 BT24 BW24 BZ24 CC24 CF24 CI24 CL24">
-    <cfRule type="expression" dxfId="133" priority="22">
+    <cfRule type="expression" dxfId="139" priority="30">
       <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BU14 BX14 CA14 CD14 CG14 CJ14 CM14 BU16 BX16 CA16 CD16 CG16 CJ16 CM16 BU18 BX18 CA18 CD18 CG18 CJ18 CM18 BU20 BX20 CA20 CD20 CG20 CJ20 CM20 BU22 BX22 CA22 CD22 CG22 CJ22 CM22 BU24 BX24 CA24 CD24 CG24 CJ24 CM24">
-    <cfRule type="expression" dxfId="134" priority="23">
+    <cfRule type="expression" dxfId="140" priority="31">
       <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BV14 BY14 CB14 CE14 CH14 CK14 CN14 BV16 BY16 CB16 CE16 CH16 CK16 CN16 BV18 BY18 CB18 CE18 CH18 CK18 CN18 BV20 BY20 CB20 CE20 CH20 CK20 CN20 BV22 BY22 CB22 CE22 CH22 CK22 CN22 BV24 BY24 CB24 CE24 CH24 CK24 CN24">
-    <cfRule type="expression" dxfId="135" priority="24">
+    <cfRule type="expression" dxfId="141" priority="32">
       <formula>AND(ISNUMBER(BT13),DATE(Planungsjahr,4,BT13)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29 F29 I29 L29 O29 R29 U29 C31 F31 I31 L31 O31 R31 U31 C33 F33 I33 L33 O33 R33 U33 C35 F35 I35 L35 O35 R35 U35 C37 F37 I37 L37 O37 R37 U37 C39 F39 I39 L39 O39 R39 U39">
-    <cfRule type="expression" dxfId="130" priority="25">
+    <cfRule type="expression" dxfId="136" priority="33">
       <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D29 G29 J29 M29 P29 S29 V29 D31 G31 J31 M31 P31 S31 V31 D33 G33 J33 M33 P33 S33 V33 D35 G35 J35 M35 P35 S35 V35 D37 G37 J37 M37 P37 S37 V37 D39 G39 J39 M39 P39 S39 V39">
-    <cfRule type="expression" dxfId="131" priority="26">
+  <conditionalFormatting sqref="C28 F28 I28 L28 O28 R28 U28 C30 F30 I30 L30 O30 R30 U30 C32 F32 I32 L32 O32 R32 U32 C34 F34 I34 L34 O34 R34 U34 C36 F36 I36 L36 O36 R36 U36 C38 F38 I38 L38 O38 R38 U38">
+    <cfRule type="expression" dxfId="137" priority="34">
       <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E29 H29 K29 N29 Q29 T29 W29 E31 H31 K31 N31 Q31 T31 W31 E33 H33 K33 N33 Q33 T33 W33 E35 H35 K35 N35 Q35 T35 W35 E37 H37 K37 N37 Q37 T37 W37 E39 H39 K39 N39 Q39 T39 W39">
-    <cfRule type="expression" dxfId="132" priority="27">
+  <conditionalFormatting sqref="D28 G28 J28 M28 P28 S28 V28 D30 G30 J30 M30 P30 S30 V30 D32 G32 J32 M32 P32 S32 V32 D34 G34 J34 M34 P34 S34 V34 D36 G36 J36 M36 P36 S36 V36 D38 G38 J38 M38 P38 S38 V38">
+    <cfRule type="expression" dxfId="137" priority="35">
+      <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28 H28 K28 N28 Q28 T28 W28 E30 H30 K30 N30 Q30 T30 W30 E32 H32 K32 N32 Q32 T32 W32 E34 H34 K34 N34 Q34 T34 W34 E36 H36 K36 N36 Q36 T36 W36 E38 H38 K38 N38 Q38 T38 W38">
+    <cfRule type="expression" dxfId="137" priority="36">
+      <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F29 I29 L29 O29 R29 U29 X29 F31 I31 L31 O31 R31 U31 X31 F33 I33 L33 O33 R33 U33 X33 F35 I35 L35 O35 R35 U35 X35 F37 I37 L37 O37 R37 U37 X37 F39 I39 L39 O39 R39 U39 X39">
+    <cfRule type="expression" dxfId="138" priority="37">
       <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C30 F30 I30 L30 O30 R30 U30 C32 F32 I32 L32 O32 R32 U32 C34 F34 I34 L34 O34 R34 U34 C36 F36 I36 L36 O36 R36 U36 C38 F38 I38 L38 O38 R38 U38 C40 F40 I40 L40 O40 R40 U40">
-    <cfRule type="expression" dxfId="133" priority="28">
+    <cfRule type="expression" dxfId="139" priority="38">
       <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D30 G30 J30 M30 P30 S30 V30 D32 G32 J32 M32 P32 S32 V32 D34 G34 J34 M34 P34 S34 V34 D36 G36 J36 M36 P36 S36 V36 D38 G38 J38 M38 P38 S38 V38 D40 G40 J40 M40 P40 S40 V40">
-    <cfRule type="expression" dxfId="134" priority="29">
+    <cfRule type="expression" dxfId="140" priority="39">
       <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30 H30 K30 N30 Q30 T30 W30 E32 H32 K32 N32 Q32 T32 W32 E34 H34 K34 N34 Q34 T34 W34 E36 H36 K36 N36 Q36 T36 W36 E38 H38 K38 N38 Q38 T38 W38 E40 H40 K40 N40 Q40 T40 W40">
-    <cfRule type="expression" dxfId="135" priority="30">
+    <cfRule type="expression" dxfId="141" priority="40">
       <formula>AND(ISNUMBER(C29),DATE(Planungsjahr,5,C29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z29 AC29 AF29 AI29 AL29 AO29 AR29 Z31 AC31 AF31 AI31 AL31 AO31 AR31 Z33 AC33 AF33 AI33 AL33 AO33 AR33 Z35 AC35 AF35 AI35 AL35 AO35 AR35 Z37 AC37 AF37 AI37 AL37 AO37 AR37 Z39 AC39 AF39 AI39 AL39 AO39 AR39">
-    <cfRule type="expression" dxfId="130" priority="31">
+    <cfRule type="expression" dxfId="136" priority="41">
       <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA29 AD29 AG29 AJ29 AM29 AP29 AS29 AA31 AD31 AG31 AJ31 AM31 AP31 AS31 AA33 AD33 AG33 AJ33 AM33 AP33 AS33 AA35 AD35 AG35 AJ35 AM35 AP35 AS35 AA37 AD37 AG37 AJ37 AM37 AP37 AS37 AA39 AD39 AG39 AJ39 AM39 AP39 AS39">
-    <cfRule type="expression" dxfId="131" priority="32">
+  <conditionalFormatting sqref="Z28 AC28 AF28 AI28 AL28 AO28 AR28 Z30 AC30 AF30 AI30 AL30 AO30 AR30 Z32 AC32 AF32 AI32 AL32 AO32 AR32 Z34 AC34 AF34 AI34 AL34 AO34 AR34 Z36 AC36 AF36 AI36 AL36 AO36 AR36 Z38 AC38 AF38 AI38 AL38 AO38 AR38">
+    <cfRule type="expression" dxfId="137" priority="42">
       <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB29 AE29 AH29 AK29 AN29 AQ29 AT29 AB31 AE31 AH31 AK31 AN31 AQ31 AT31 AB33 AE33 AH33 AK33 AN33 AQ33 AT33 AB35 AE35 AH35 AK35 AN35 AQ35 AT35 AB37 AE37 AH37 AK37 AN37 AQ37 AT37 AB39 AE39 AH39 AK39 AN39 AQ39 AT39">
-    <cfRule type="expression" dxfId="132" priority="33">
+  <conditionalFormatting sqref="AA28 AD28 AG28 AJ28 AM28 AP28 AS28 AA30 AD30 AG30 AJ30 AM30 AP30 AS30 AA32 AD32 AG32 AJ32 AM32 AP32 AS32 AA34 AD34 AG34 AJ34 AM34 AP34 AS34 AA36 AD36 AG36 AJ36 AM36 AP36 AS36 AA38 AD38 AG38 AJ38 AM38 AP38 AS38">
+    <cfRule type="expression" dxfId="137" priority="43">
+      <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB28 AE28 AH28 AK28 AN28 AQ28 AT28 AB30 AE30 AH30 AK30 AN30 AQ30 AT30 AB32 AE32 AH32 AK32 AN32 AQ32 AT32 AB34 AE34 AH34 AK34 AN34 AQ34 AT34 AB36 AE36 AH36 AK36 AN36 AQ36 AT36 AB38 AE38 AH38 AK38 AN38 AQ38 AT38">
+    <cfRule type="expression" dxfId="137" priority="44">
+      <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC29 AF29 AI29 AL29 AO29 AR29 AU29 AC31 AF31 AI31 AL31 AO31 AR31 AU31 AC33 AF33 AI33 AL33 AO33 AR33 AU33 AC35 AF35 AI35 AL35 AO35 AR35 AU35 AC37 AF37 AI37 AL37 AO37 AR37 AU37 AC39 AF39 AI39 AL39 AO39 AR39 AU39">
+    <cfRule type="expression" dxfId="138" priority="45">
       <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z30 AC30 AF30 AI30 AL30 AO30 AR30 Z32 AC32 AF32 AI32 AL32 AO32 AR32 Z34 AC34 AF34 AI34 AL34 AO34 AR34 Z36 AC36 AF36 AI36 AL36 AO36 AR36 Z38 AC38 AF38 AI38 AL38 AO38 AR38 Z40 AC40 AF40 AI40 AL40 AO40 AR40">
-    <cfRule type="expression" dxfId="133" priority="34">
+    <cfRule type="expression" dxfId="139" priority="46">
       <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA30 AD30 AG30 AJ30 AM30 AP30 AS30 AA32 AD32 AG32 AJ32 AM32 AP32 AS32 AA34 AD34 AG34 AJ34 AM34 AP34 AS34 AA36 AD36 AG36 AJ36 AM36 AP36 AS36 AA38 AD38 AG38 AJ38 AM38 AP38 AS38 AA40 AD40 AG40 AJ40 AM40 AP40 AS40">
-    <cfRule type="expression" dxfId="134" priority="35">
+    <cfRule type="expression" dxfId="140" priority="47">
       <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB30 AE30 AH30 AK30 AN30 AQ30 AT30 AB32 AE32 AH32 AK32 AN32 AQ32 AT32 AB34 AE34 AH34 AK34 AN34 AQ34 AT34 AB36 AE36 AH36 AK36 AN36 AQ36 AT36 AB38 AE38 AH38 AK38 AN38 AQ38 AT38 AB40 AE40 AH40 AK40 AN40 AQ40 AT40">
-    <cfRule type="expression" dxfId="135" priority="36">
+    <cfRule type="expression" dxfId="141" priority="48">
       <formula>AND(ISNUMBER(Z29),DATE(Planungsjahr,6,Z29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW29 AZ29 BC29 BF29 BI29 BL29 BO29 AW31 AZ31 BC31 BF31 BI31 BL31 BO31 AW33 AZ33 BC33 BF33 BI33 BL33 BO33 AW35 AZ35 BC35 BF35 BI35 BL35 BO35 AW37 AZ37 BC37 BF37 BI37 BL37 BO37 AW39 AZ39 BC39 BF39 BI39 BL39 BO39">
-    <cfRule type="expression" dxfId="130" priority="37">
+    <cfRule type="expression" dxfId="136" priority="49">
       <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AX29 BA29 BD29 BG29 BJ29 BM29 BP29 AX31 BA31 BD31 BG31 BJ31 BM31 BP31 AX33 BA33 BD33 BG33 BJ33 BM33 BP33 AX35 BA35 BD35 BG35 BJ35 BM35 BP35 AX37 BA37 BD37 BG37 BJ37 BM37 BP37 AX39 BA39 BD39 BG39 BJ39 BM39 BP39">
-    <cfRule type="expression" dxfId="131" priority="38">
+  <conditionalFormatting sqref="AW28 AZ28 BC28 BF28 BI28 BL28 BO28 AW30 AZ30 BC30 BF30 BI30 BL30 BO30 AW32 AZ32 BC32 BF32 BI32 BL32 BO32 AW34 AZ34 BC34 BF34 BI34 BL34 BO34 AW36 AZ36 BC36 BF36 BI36 BL36 BO36 AW38 AZ38 BC38 BF38 BI38 BL38 BO38">
+    <cfRule type="expression" dxfId="137" priority="50">
       <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AY29 BB29 BE29 BH29 BK29 BN29 BQ29 AY31 BB31 BE31 BH31 BK31 BN31 BQ31 AY33 BB33 BE33 BH33 BK33 BN33 BQ33 AY35 BB35 BE35 BH35 BK35 BN35 BQ35 AY37 BB37 BE37 BH37 BK37 BN37 BQ37 AY39 BB39 BE39 BH39 BK39 BN39 BQ39">
-    <cfRule type="expression" dxfId="132" priority="39">
+  <conditionalFormatting sqref="AX28 BA28 BD28 BG28 BJ28 BM28 BP28 AX30 BA30 BD30 BG30 BJ30 BM30 BP30 AX32 BA32 BD32 BG32 BJ32 BM32 BP32 AX34 BA34 BD34 BG34 BJ34 BM34 BP34 AX36 BA36 BD36 BG36 BJ36 BM36 BP36 AX38 BA38 BD38 BG38 BJ38 BM38 BP38">
+    <cfRule type="expression" dxfId="137" priority="51">
+      <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AY28 BB28 BE28 BH28 BK28 BN28 BQ28 AY30 BB30 BE30 BH30 BK30 BN30 BQ30 AY32 BB32 BE32 BH32 BK32 BN32 BQ32 AY34 BB34 BE34 BH34 BK34 BN34 BQ34 AY36 BB36 BE36 BH36 BK36 BN36 BQ36 AY38 BB38 BE38 BH38 BK38 BN38 BQ38">
+    <cfRule type="expression" dxfId="137" priority="52">
+      <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AZ29 BC29 BF29 BI29 BL29 BO29 BR29 AZ31 BC31 BF31 BI31 BL31 BO31 BR31 AZ33 BC33 BF33 BI33 BL33 BO33 BR33 AZ35 BC35 BF35 BI35 BL35 BO35 BR35 AZ37 BC37 BF37 BI37 BL37 BO37 BR37 AZ39 BC39 BF39 BI39 BL39 BO39 BR39">
+    <cfRule type="expression" dxfId="138" priority="53">
       <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW30 AZ30 BC30 BF30 BI30 BL30 BO30 AW32 AZ32 BC32 BF32 BI32 BL32 BO32 AW34 AZ34 BC34 BF34 BI34 BL34 BO34 AW36 AZ36 BC36 BF36 BI36 BL36 BO36 AW38 AZ38 BC38 BF38 BI38 BL38 BO38 AW40 AZ40 BC40 BF40 BI40 BL40 BO40">
-    <cfRule type="expression" dxfId="133" priority="40">
+    <cfRule type="expression" dxfId="139" priority="54">
       <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AX30 BA30 BD30 BG30 BJ30 BM30 BP30 AX32 BA32 BD32 BG32 BJ32 BM32 BP32 AX34 BA34 BD34 BG34 BJ34 BM34 BP34 AX36 BA36 BD36 BG36 BJ36 BM36 BP36 AX38 BA38 BD38 BG38 BJ38 BM38 BP38 AX40 BA40 BD40 BG40 BJ40 BM40 BP40">
-    <cfRule type="expression" dxfId="134" priority="41">
+    <cfRule type="expression" dxfId="140" priority="55">
       <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AY30 BB30 BE30 BH30 BK30 BN30 BQ30 AY32 BB32 BE32 BH32 BK32 BN32 BQ32 AY34 BB34 BE34 BH34 BK34 BN34 BQ34 AY36 BB36 BE36 BH36 BK36 BN36 BQ36 AY38 BB38 BE38 BH38 BK38 BN38 BQ38 AY40 BB40 BE40 BH40 BK40 BN40 BQ40">
-    <cfRule type="expression" dxfId="135" priority="42">
+    <cfRule type="expression" dxfId="141" priority="56">
       <formula>AND(ISNUMBER(AW29),DATE(Planungsjahr,7,AW29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT29 BW29 BZ29 CC29 CF29 CI29 CL29 BT31 BW31 BZ31 CC31 CF31 CI31 CL31 BT33 BW33 BZ33 CC33 CF33 CI33 CL33 BT35 BW35 BZ35 CC35 CF35 CI35 CL35 BT37 BW37 BZ37 CC37 CF37 CI37 CL37 BT39 BW39 BZ39 CC39 CF39 CI39 CL39">
-    <cfRule type="expression" dxfId="130" priority="43">
+    <cfRule type="expression" dxfId="136" priority="57">
       <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BU29 BX29 CA29 CD29 CG29 CJ29 CM29 BU31 BX31 CA31 CD31 CG31 CJ31 CM31 BU33 BX33 CA33 CD33 CG33 CJ33 CM33 BU35 BX35 CA35 CD35 CG35 CJ35 CM35 BU37 BX37 CA37 CD37 CG37 CJ37 CM37 BU39 BX39 CA39 CD39 CG39 CJ39 CM39">
-    <cfRule type="expression" dxfId="131" priority="44">
+  <conditionalFormatting sqref="BT28 BW28 BZ28 CC28 CF28 CI28 CL28 BT30 BW30 BZ30 CC30 CF30 CI30 CL30 BT32 BW32 BZ32 CC32 CF32 CI32 CL32 BT34 BW34 BZ34 CC34 CF34 CI34 CL34 BT36 BW36 BZ36 CC36 CF36 CI36 CL36 BT38 BW38 BZ38 CC38 CF38 CI38 CL38">
+    <cfRule type="expression" dxfId="137" priority="58">
       <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BV29 BY29 CB29 CE29 CH29 CK29 CN29 BV31 BY31 CB31 CE31 CH31 CK31 CN31 BV33 BY33 CB33 CE33 CH33 CK33 CN33 BV35 BY35 CB35 CE35 CH35 CK35 CN35 BV37 BY37 CB37 CE37 CH37 CK37 CN37 BV39 BY39 CB39 CE39 CH39 CK39 CN39">
-    <cfRule type="expression" dxfId="132" priority="45">
+  <conditionalFormatting sqref="BU28 BX28 CA28 CD28 CG28 CJ28 CM28 BU30 BX30 CA30 CD30 CG30 CJ30 CM30 BU32 BX32 CA32 CD32 CG32 CJ32 CM32 BU34 BX34 CA34 CD34 CG34 CJ34 CM34 BU36 BX36 CA36 CD36 CG36 CJ36 CM36 BU38 BX38 CA38 CD38 CG38 CJ38 CM38">
+    <cfRule type="expression" dxfId="137" priority="59">
+      <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BV28 BY28 CB28 CE28 CH28 CK28 CN28 BV30 BY30 CB30 CE30 CH30 CK30 CN30 BV32 BY32 CB32 CE32 CH32 CK32 CN32 BV34 BY34 CB34 CE34 CH34 CK34 CN34 BV36 BY36 CB36 CE36 CH36 CK36 CN36 BV38 BY38 CB38 CE38 CH38 CK38 CN38">
+    <cfRule type="expression" dxfId="137" priority="60">
+      <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BW29 BZ29 CC29 CF29 CI29 CL29 CO29 BW31 BZ31 CC31 CF31 CI31 CL31 CO31 BW33 BZ33 CC33 CF33 CI33 CL33 CO33 BW35 BZ35 CC35 CF35 CI35 CL35 CO35 BW37 BZ37 CC37 CF37 CI37 CL37 CO37 BW39 BZ39 CC39 CF39 CI39 CL39 CO39">
+    <cfRule type="expression" dxfId="138" priority="61">
       <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT30 BW30 BZ30 CC30 CF30 CI30 CL30 BT32 BW32 BZ32 CC32 CF32 CI32 CL32 BT34 BW34 BZ34 CC34 CF34 CI34 CL34 BT36 BW36 BZ36 CC36 CF36 CI36 CL36 BT38 BW38 BZ38 CC38 CF38 CI38 CL38 BT40 BW40 BZ40 CC40 CF40 CI40 CL40">
-    <cfRule type="expression" dxfId="133" priority="46">
+    <cfRule type="expression" dxfId="139" priority="62">
       <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BU30 BX30 CA30 CD30 CG30 CJ30 CM30 BU32 BX32 CA32 CD32 CG32 CJ32 CM32 BU34 BX34 CA34 CD34 CG34 CJ34 CM34 BU36 BX36 CA36 CD36 CG36 CJ36 CM36 BU38 BX38 CA38 CD38 CG38 CJ38 CM38 BU40 BX40 CA40 CD40 CG40 CJ40 CM40">
-    <cfRule type="expression" dxfId="134" priority="47">
+    <cfRule type="expression" dxfId="140" priority="63">
       <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BV30 BY30 CB30 CE30 CH30 CK30 CN30 BV32 BY32 CB32 CE32 CH32 CK32 CN32 BV34 BY34 CB34 CE34 CH34 CK34 CN34 BV36 BY36 CB36 CE36 CH36 CK36 CN36 BV38 BY38 CB38 CE38 CH38 CK38 CN38 BV40 BY40 CB40 CE40 CH40 CK40 CN40">
-    <cfRule type="expression" dxfId="135" priority="48">
+    <cfRule type="expression" dxfId="141" priority="64">
       <formula>AND(ISNUMBER(BT29),DATE(Planungsjahr,8,BT29)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45 F45 I45 L45 O45 R45 U45 C47 F47 I47 L47 O47 R47 U47 C49 F49 I49 L49 O49 R49 U49 C51 F51 I51 L51 O51 R51 U51 C53 F53 I53 L53 O53 R53 U53 C55 F55 I55 L55 O55 R55 U55">
-    <cfRule type="expression" dxfId="130" priority="49">
+    <cfRule type="expression" dxfId="136" priority="65">
       <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D45 G45 J45 M45 P45 S45 V45 D47 G47 J47 M47 P47 S47 V47 D49 G49 J49 M49 P49 S49 V49 D51 G51 J51 M51 P51 S51 V51 D53 G53 J53 M53 P53 S53 V53 D55 G55 J55 M55 P55 S55 V55">
-    <cfRule type="expression" dxfId="131" priority="50">
+  <conditionalFormatting sqref="C44 F44 I44 L44 O44 R44 U44 C46 F46 I46 L46 O46 R46 U46 C48 F48 I48 L48 O48 R48 U48 C50 F50 I50 L50 O50 R50 U50 C52 F52 I52 L52 O52 R52 U52 C54 F54 I54 L54 O54 R54 U54">
+    <cfRule type="expression" dxfId="137" priority="66">
       <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E45 H45 K45 N45 Q45 T45 W45 E47 H47 K47 N47 Q47 T47 W47 E49 H49 K49 N49 Q49 T49 W49 E51 H51 K51 N51 Q51 T51 W51 E53 H53 K53 N53 Q53 T53 W53 E55 H55 K55 N55 Q55 T55 W55">
-    <cfRule type="expression" dxfId="132" priority="51">
+  <conditionalFormatting sqref="D44 G44 J44 M44 P44 S44 V44 D46 G46 J46 M46 P46 S46 V46 D48 G48 J48 M48 P48 S48 V48 D50 G50 J50 M50 P50 S50 V50 D52 G52 J52 M52 P52 S52 V52 D54 G54 J54 M54 P54 S54 V54">
+    <cfRule type="expression" dxfId="137" priority="67">
+      <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E44 H44 K44 N44 Q44 T44 W44 E46 H46 K46 N46 Q46 T46 W46 E48 H48 K48 N48 Q48 T48 W48 E50 H50 K50 N50 Q50 T50 W50 E52 H52 K52 N52 Q52 T52 W52 E54 H54 K54 N54 Q54 T54 W54">
+    <cfRule type="expression" dxfId="137" priority="68">
+      <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F45 I45 L45 O45 R45 U45 X45 F47 I47 L47 O47 R47 U47 X47 F49 I49 L49 O49 R49 U49 X49 F51 I51 L51 O51 R51 U51 X51 F53 I53 L53 O53 R53 U53 X53 F55 I55 L55 O55 R55 U55 X55">
+    <cfRule type="expression" dxfId="138" priority="69">
       <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C46 F46 I46 L46 O46 R46 U46 C48 F48 I48 L48 O48 R48 U48 C50 F50 I50 L50 O50 R50 U50 C52 F52 I52 L52 O52 R52 U52 C54 F54 I54 L54 O54 R54 U54 C56 F56 I56 L56 O56 R56 U56">
-    <cfRule type="expression" dxfId="133" priority="52">
+    <cfRule type="expression" dxfId="139" priority="70">
       <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D46 G46 J46 M46 P46 S46 V46 D48 G48 J48 M48 P48 S48 V48 D50 G50 J50 M50 P50 S50 V50 D52 G52 J52 M52 P52 S52 V52 D54 G54 J54 M54 P54 S54 V54 D56 G56 J56 M56 P56 S56 V56">
-    <cfRule type="expression" dxfId="134" priority="53">
+    <cfRule type="expression" dxfId="140" priority="71">
       <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E46 H46 K46 N46 Q46 T46 W46 E48 H48 K48 N48 Q48 T48 W48 E50 H50 K50 N50 Q50 T50 W50 E52 H52 K52 N52 Q52 T52 W52 E54 H54 K54 N54 Q54 T54 W54 E56 H56 K56 N56 Q56 T56 W56">
-    <cfRule type="expression" dxfId="135" priority="54">
+    <cfRule type="expression" dxfId="141" priority="72">
       <formula>AND(ISNUMBER(C45),DATE(Planungsjahr,9,C45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z45 AC45 AF45 AI45 AL45 AO45 AR45 Z47 AC47 AF47 AI47 AL47 AO47 AR47 Z49 AC49 AF49 AI49 AL49 AO49 AR49 Z51 AC51 AF51 AI51 AL51 AO51 AR51 Z53 AC53 AF53 AI53 AL53 AO53 AR53 Z55 AC55 AF55 AI55 AL55 AO55 AR55">
-    <cfRule type="expression" dxfId="130" priority="55">
+    <cfRule type="expression" dxfId="136" priority="73">
       <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA45 AD45 AG45 AJ45 AM45 AP45 AS45 AA47 AD47 AG47 AJ47 AM47 AP47 AS47 AA49 AD49 AG49 AJ49 AM49 AP49 AS49 AA51 AD51 AG51 AJ51 AM51 AP51 AS51 AA53 AD53 AG53 AJ53 AM53 AP53 AS53 AA55 AD55 AG55 AJ55 AM55 AP55 AS55">
-    <cfRule type="expression" dxfId="131" priority="56">
+  <conditionalFormatting sqref="Z44 AC44 AF44 AI44 AL44 AO44 AR44 Z46 AC46 AF46 AI46 AL46 AO46 AR46 Z48 AC48 AF48 AI48 AL48 AO48 AR48 Z50 AC50 AF50 AI50 AL50 AO50 AR50 Z52 AC52 AF52 AI52 AL52 AO52 AR52 Z54 AC54 AF54 AI54 AL54 AO54 AR54">
+    <cfRule type="expression" dxfId="137" priority="74">
       <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB45 AE45 AH45 AK45 AN45 AQ45 AT45 AB47 AE47 AH47 AK47 AN47 AQ47 AT47 AB49 AE49 AH49 AK49 AN49 AQ49 AT49 AB51 AE51 AH51 AK51 AN51 AQ51 AT51 AB53 AE53 AH53 AK53 AN53 AQ53 AT53 AB55 AE55 AH55 AK55 AN55 AQ55 AT55">
-    <cfRule type="expression" dxfId="132" priority="57">
+  <conditionalFormatting sqref="AA44 AD44 AG44 AJ44 AM44 AP44 AS44 AA46 AD46 AG46 AJ46 AM46 AP46 AS46 AA48 AD48 AG48 AJ48 AM48 AP48 AS48 AA50 AD50 AG50 AJ50 AM50 AP50 AS50 AA52 AD52 AG52 AJ52 AM52 AP52 AS52 AA54 AD54 AG54 AJ54 AM54 AP54 AS54">
+    <cfRule type="expression" dxfId="137" priority="75">
+      <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB44 AE44 AH44 AK44 AN44 AQ44 AT44 AB46 AE46 AH46 AK46 AN46 AQ46 AT46 AB48 AE48 AH48 AK48 AN48 AQ48 AT48 AB50 AE50 AH50 AK50 AN50 AQ50 AT50 AB52 AE52 AH52 AK52 AN52 AQ52 AT52 AB54 AE54 AH54 AK54 AN54 AQ54 AT54">
+    <cfRule type="expression" dxfId="137" priority="76">
+      <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC45 AF45 AI45 AL45 AO45 AR45 AU45 AC47 AF47 AI47 AL47 AO47 AR47 AU47 AC49 AF49 AI49 AL49 AO49 AR49 AU49 AC51 AF51 AI51 AL51 AO51 AR51 AU51 AC53 AF53 AI53 AL53 AO53 AR53 AU53 AC55 AF55 AI55 AL55 AO55 AR55 AU55">
+    <cfRule type="expression" dxfId="138" priority="77">
       <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z46 AC46 AF46 AI46 AL46 AO46 AR46 Z48 AC48 AF48 AI48 AL48 AO48 AR48 Z50 AC50 AF50 AI50 AL50 AO50 AR50 Z52 AC52 AF52 AI52 AL52 AO52 AR52 Z54 AC54 AF54 AI54 AL54 AO54 AR54 Z56 AC56 AF56 AI56 AL56 AO56 AR56">
-    <cfRule type="expression" dxfId="133" priority="58">
+    <cfRule type="expression" dxfId="139" priority="78">
       <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA46 AD46 AG46 AJ46 AM46 AP46 AS46 AA48 AD48 AG48 AJ48 AM48 AP48 AS48 AA50 AD50 AG50 AJ50 AM50 AP50 AS50 AA52 AD52 AG52 AJ52 AM52 AP52 AS52 AA54 AD54 AG54 AJ54 AM54 AP54 AS54 AA56 AD56 AG56 AJ56 AM56 AP56 AS56">
-    <cfRule type="expression" dxfId="134" priority="59">
+    <cfRule type="expression" dxfId="140" priority="79">
       <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB46 AE46 AH46 AK46 AN46 AQ46 AT46 AB48 AE48 AH48 AK48 AN48 AQ48 AT48 AB50 AE50 AH50 AK50 AN50 AQ50 AT50 AB52 AE52 AH52 AK52 AN52 AQ52 AT52 AB54 AE54 AH54 AK54 AN54 AQ54 AT54 AB56 AE56 AH56 AK56 AN56 AQ56 AT56">
-    <cfRule type="expression" dxfId="135" priority="60">
+    <cfRule type="expression" dxfId="141" priority="80">
       <formula>AND(ISNUMBER(Z45),DATE(Planungsjahr,10,Z45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW45 AZ45 BC45 BF45 BI45 BL45 BO45 AW47 AZ47 BC47 BF47 BI47 BL47 BO47 AW49 AZ49 BC49 BF49 BI49 BL49 BO49 AW51 AZ51 BC51 BF51 BI51 BL51 BO51 AW53 AZ53 BC53 BF53 BI53 BL53 BO53 AW55 AZ55 BC55 BF55 BI55 BL55 BO55">
-    <cfRule type="expression" dxfId="130" priority="61">
+    <cfRule type="expression" dxfId="136" priority="81">
       <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AX45 BA45 BD45 BG45 BJ45 BM45 BP45 AX47 BA47 BD47 BG47 BJ47 BM47 BP47 AX49 BA49 BD49 BG49 BJ49 BM49 BP49 AX51 BA51 BD51 BG51 BJ51 BM51 BP51 AX53 BA53 BD53 BG53 BJ53 BM53 BP53 AX55 BA55 BD55 BG55 BJ55 BM55 BP55">
-    <cfRule type="expression" dxfId="131" priority="62">
+  <conditionalFormatting sqref="AW44 AZ44 BC44 BF44 BI44 BL44 BO44 AW46 AZ46 BC46 BF46 BI46 BL46 BO46 AW48 AZ48 BC48 BF48 BI48 BL48 BO48 AW50 AZ50 BC50 BF50 BI50 BL50 BO50 AW52 AZ52 BC52 BF52 BI52 BL52 BO52 AW54 AZ54 BC54 BF54 BI54 BL54 BO54">
+    <cfRule type="expression" dxfId="137" priority="82">
       <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AY45 BB45 BE45 BH45 BK45 BN45 BQ45 AY47 BB47 BE47 BH47 BK47 BN47 BQ47 AY49 BB49 BE49 BH49 BK49 BN49 BQ49 AY51 BB51 BE51 BH51 BK51 BN51 BQ51 AY53 BB53 BE53 BH53 BK53 BN53 BQ53 AY55 BB55 BE55 BH55 BK55 BN55 BQ55">
-    <cfRule type="expression" dxfId="132" priority="63">
+  <conditionalFormatting sqref="AX44 BA44 BD44 BG44 BJ44 BM44 BP44 AX46 BA46 BD46 BG46 BJ46 BM46 BP46 AX48 BA48 BD48 BG48 BJ48 BM48 BP48 AX50 BA50 BD50 BG50 BJ50 BM50 BP50 AX52 BA52 BD52 BG52 BJ52 BM52 BP52 AX54 BA54 BD54 BG54 BJ54 BM54 BP54">
+    <cfRule type="expression" dxfId="137" priority="83">
+      <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AY44 BB44 BE44 BH44 BK44 BN44 BQ44 AY46 BB46 BE46 BH46 BK46 BN46 BQ46 AY48 BB48 BE48 BH48 BK48 BN48 BQ48 AY50 BB50 BE50 BH50 BK50 BN50 BQ50 AY52 BB52 BE52 BH52 BK52 BN52 BQ52 AY54 BB54 BE54 BH54 BK54 BN54 BQ54">
+    <cfRule type="expression" dxfId="137" priority="84">
+      <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AZ45 BC45 BF45 BI45 BL45 BO45 BR45 AZ47 BC47 BF47 BI47 BL47 BO47 BR47 AZ49 BC49 BF49 BI49 BL49 BO49 BR49 AZ51 BC51 BF51 BI51 BL51 BO51 BR51 AZ53 BC53 BF53 BI53 BL53 BO53 BR53 AZ55 BC55 BF55 BI55 BL55 BO55 BR55">
+    <cfRule type="expression" dxfId="138" priority="85">
       <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW46 AZ46 BC46 BF46 BI46 BL46 BO46 AW48 AZ48 BC48 BF48 BI48 BL48 BO48 AW50 AZ50 BC50 BF50 BI50 BL50 BO50 AW52 AZ52 BC52 BF52 BI52 BL52 BO52 AW54 AZ54 BC54 BF54 BI54 BL54 BO54 AW56 AZ56 BC56 BF56 BI56 BL56 BO56">
-    <cfRule type="expression" dxfId="133" priority="64">
+    <cfRule type="expression" dxfId="139" priority="86">
       <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AX46 BA46 BD46 BG46 BJ46 BM46 BP46 AX48 BA48 BD48 BG48 BJ48 BM48 BP48 AX50 BA50 BD50 BG50 BJ50 BM50 BP50 AX52 BA52 BD52 BG52 BJ52 BM52 BP52 AX54 BA54 BD54 BG54 BJ54 BM54 BP54 AX56 BA56 BD56 BG56 BJ56 BM56 BP56">
-    <cfRule type="expression" dxfId="134" priority="65">
+    <cfRule type="expression" dxfId="140" priority="87">
       <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AY46 BB46 BE46 BH46 BK46 BN46 BQ46 AY48 BB48 BE48 BH48 BK48 BN48 BQ48 AY50 BB50 BE50 BH50 BK50 BN50 BQ50 AY52 BB52 BE52 BH52 BK52 BN52 BQ52 AY54 BB54 BE54 BH54 BK54 BN54 BQ54 AY56 BB56 BE56 BH56 BK56 BN56 BQ56">
-    <cfRule type="expression" dxfId="135" priority="66">
+    <cfRule type="expression" dxfId="141" priority="88">
       <formula>AND(ISNUMBER(AW45),DATE(Planungsjahr,11,AW45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT45 BW45 BZ45 CC45 CF45 CI45 CL45 BT47 BW47 BZ47 CC47 CF47 CI47 CL47 BT49 BW49 BZ49 CC49 CF49 CI49 CL49 BT51 BW51 BZ51 CC51 CF51 CI51 CL51 BT53 BW53 BZ53 CC53 CF53 CI53 CL53 BT55 BW55 BZ55 CC55 CF55 CI55 CL55">
-    <cfRule type="expression" dxfId="130" priority="67">
+    <cfRule type="expression" dxfId="136" priority="89">
       <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BU45 BX45 CA45 CD45 CG45 CJ45 CM45 BU47 BX47 CA47 CD47 CG47 CJ47 CM47 BU49 BX49 CA49 CD49 CG49 CJ49 CM49 BU51 BX51 CA51 CD51 CG51 CJ51 CM51 BU53 BX53 CA53 CD53 CG53 CJ53 CM53 BU55 BX55 CA55 CD55 CG55 CJ55 CM55">
-    <cfRule type="expression" dxfId="131" priority="68">
+  <conditionalFormatting sqref="BT44 BW44 BZ44 CC44 CF44 CI44 CL44 BT46 BW46 BZ46 CC46 CF46 CI46 CL46 BT48 BW48 BZ48 CC48 CF48 CI48 CL48 BT50 BW50 BZ50 CC50 CF50 CI50 CL50 BT52 BW52 BZ52 CC52 CF52 CI52 CL52 BT54 BW54 BZ54 CC54 CF54 CI54 CL54">
+    <cfRule type="expression" dxfId="137" priority="90">
       <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BV45 BY45 CB45 CE45 CH45 CK45 CN45 BV47 BY47 CB47 CE47 CH47 CK47 CN47 BV49 BY49 CB49 CE49 CH49 CK49 CN49 BV51 BY51 CB51 CE51 CH51 CK51 CN51 BV53 BY53 CB53 CE53 CH53 CK53 CN53 BV55 BY55 CB55 CE55 CH55 CK55 CN55">
-    <cfRule type="expression" dxfId="132" priority="69">
+  <conditionalFormatting sqref="BU44 BX44 CA44 CD44 CG44 CJ44 CM44 BU46 BX46 CA46 CD46 CG46 CJ46 CM46 BU48 BX48 CA48 CD48 CG48 CJ48 CM48 BU50 BX50 CA50 CD50 CG50 CJ50 CM50 BU52 BX52 CA52 CD52 CG52 CJ52 CM52 BU54 BX54 CA54 CD54 CG54 CJ54 CM54">
+    <cfRule type="expression" dxfId="137" priority="91">
+      <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BV44 BY44 CB44 CE44 CH44 CK44 CN44 BV46 BY46 CB46 CE46 CH46 CK46 CN46 BV48 BY48 CB48 CE48 CH48 CK48 CN48 BV50 BY50 CB50 CE50 CH50 CK50 CN50 BV52 BY52 CB52 CE52 CH52 CK52 CN52 BV54 BY54 CB54 CE54 CH54 CK54 CN54">
+    <cfRule type="expression" dxfId="137" priority="92">
+      <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BW45 BZ45 CC45 CF45 CI45 CL45 CO45 BW47 BZ47 CC47 CF47 CI47 CL47 CO47 BW49 BZ49 CC49 CF49 CI49 CL49 CO49 BW51 BZ51 CC51 CF51 CI51 CL51 CO51 BW53 BZ53 CC53 CF53 CI53 CL53 CO53 BW55 BZ55 CC55 CF55 CI55 CL55 CO55">
+    <cfRule type="expression" dxfId="138" priority="93">
       <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT46 BW46 BZ46 CC46 CF46 CI46 CL46 BT48 BW48 BZ48 CC48 CF48 CI48 CL48 BT50 BW50 BZ50 CC50 CF50 CI50 CL50 BT52 BW52 BZ52 CC52 CF52 CI52 CL52 BT54 BW54 BZ54 CC54 CF54 CI54 CL54 BT56 BW56 BZ56 CC56 CF56 CI56 CL56">
-    <cfRule type="expression" dxfId="133" priority="70">
+    <cfRule type="expression" dxfId="139" priority="94">
       <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BU46 BX46 CA46 CD46 CG46 CJ46 CM46 BU48 BX48 CA48 CD48 CG48 CJ48 CM48 BU50 BX50 CA50 CD50 CG50 CJ50 CM50 BU52 BX52 CA52 CD52 CG52 CJ52 CM52 BU54 BX54 CA54 CD54 CG54 CJ54 CM54 BU56 BX56 CA56 CD56 CG56 CJ56 CM56">
-    <cfRule type="expression" dxfId="134" priority="71">
+    <cfRule type="expression" dxfId="140" priority="95">
       <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BV46 BY46 CB46 CE46 CH46 CK46 CN46 BV48 BY48 CB48 CE48 CH48 CK48 CN48 BV50 BY50 CB50 CE50 CH50 CK50 CN50 BV52 BY52 CB52 CE52 CH52 CK52 CN52 BV54 BY54 CB54 CE54 CH54 CK54 CN54 BV56 BY56 CB56 CE56 CH56 CK56 CN56">
-    <cfRule type="expression" dxfId="135" priority="72">
+    <cfRule type="expression" dxfId="141" priority="96">
       <formula>AND(ISNUMBER(BT45),DATE(Planungsjahr,12,BT45)=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:W13 C15:W15 C17:W17 C19:W19 C21:W21 C23:W23">
-    <cfRule type="expression" dxfId="101" priority="202" stopIfTrue="1">
+    <cfRule type="expression" dxfId="101" priority="702" stopIfTrue="1">
       <formula>AND(ISNUMBER(C13),COUNTIF(Feiertage,DATE(Planungsjahr,1,C13))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="203" stopIfTrue="1">
+    <cfRule type="expression" dxfId="101" priority="703" stopIfTrue="1">
       <formula>AND(ISNUMBER(C13),WEEKDAY(DATE(Planungsjahr,1,C13),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14:W14 Z14:AT14 AW14:BQ14 BT14:CN14 C16:W16 Z16:AT16 AW16:BQ16 BT16:CN16 C18:W18 Z18:AT18 AW18:BQ18 BT18:CN18 C20:W20 Z20:AT20 AW20:BQ20 BT20:CN20 C22:W22 Z22:AT22 AW22:BQ22 BT22:CN22 C24:W24 Z24:AT24 AW24:BQ24 BT24:CN24 C30:W30 Z30:AT30 AW30:BQ30 BT30:CN30 C32:W32 Z32:AT32 AW32:BQ32 BT32:CN32 C34:W34 Z34:AT34 AW34:BQ34 BT34:CN34 C36:W36 Z36:AT36 AW36:BQ36 BT36:CN36 C38:W38 Z38:AT38 AW38:BQ38 BT38:CN38 C40:W40 Z40:AT40 AW40:BQ40 BT40:CN40 C46:W46 Z46:AT46 AW46:BQ46 BT46:CN46 C48:W48 Z48:AT48 AW48:BQ48 BT48:CN48 C50:W50 Z50:AT50 AW50:BQ50 BT50:CN50 C52:W52 Z52:AT52 AW52:BQ52 BT52:CN52 C54:W54 Z54:AT54 AW54:BQ54 BT54:CN54 C56:W56 Z56:AT56 AW56:BQ56 BT56:CN56">
-    <cfRule type="cellIs" dxfId="100" priority="230" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="730" stopIfTrue="1" operator="equal">
       <formula>"w"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="229" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="729" stopIfTrue="1" operator="equal">
       <formula>"h"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="228" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="728" stopIfTrue="1" operator="equal">
       <formula>"P"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="227" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="727" stopIfTrue="1" operator="equal">
       <formula>"I"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="226" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="726" stopIfTrue="1" operator="equal">
       <formula>"S"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29:W29 C31:W31 C33:W33 C35:W35 C37:W37 C39:W39">
-    <cfRule type="expression" dxfId="94" priority="210" stopIfTrue="1">
+    <cfRule type="expression" dxfId="94" priority="710" stopIfTrue="1">
       <formula>AND(ISNUMBER(C29),COUNTIF(Feiertage,DATE(Planungsjahr,5,C29))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="94" priority="211" stopIfTrue="1">
+    <cfRule type="expression" dxfId="94" priority="711" stopIfTrue="1">
       <formula>AND(ISNUMBER(C29),WEEKDAY(DATE(Planungsjahr,5,C29),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45:W45 C47:W47 C49:W49 C51:W51 C53:W53 C55:W55">
-    <cfRule type="expression" dxfId="92" priority="218" stopIfTrue="1">
+    <cfRule type="expression" dxfId="92" priority="718" stopIfTrue="1">
       <formula>AND(ISNUMBER(C45),COUNTIF(Feiertage,DATE(Planungsjahr,9,C45))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="92" priority="219" stopIfTrue="1">
+    <cfRule type="expression" dxfId="92" priority="719" stopIfTrue="1">
       <formula>AND(ISNUMBER(C45),WEEKDAY(DATE(Planungsjahr,9,C45),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z62:Z81">
-    <cfRule type="expression" dxfId="0" priority="231">
+    <cfRule type="expression" dxfId="0" priority="731">
       <formula>AND(ISNUMBER(Z62),YEAR(Z62)&lt;&gt;Planungsjahr)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z13:AT13 Z15:AT15 Z17:AT17 Z19:AT19 Z21:AT21 Z23:AT23">
-    <cfRule type="expression" dxfId="90" priority="204" stopIfTrue="1">
+    <cfRule type="expression" dxfId="90" priority="704" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z13),COUNTIF(Feiertage,DATE(Planungsjahr,2,Z13))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="90" priority="205" stopIfTrue="1">
+    <cfRule type="expression" dxfId="90" priority="705" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z13),WEEKDAY(DATE(Planungsjahr,2,Z13),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z29:AT29 Z31:AT31 Z33:AT33 Z35:AT35 Z37:AT37 Z39:AT39">
-    <cfRule type="expression" dxfId="88" priority="212" stopIfTrue="1">
+    <cfRule type="expression" dxfId="88" priority="712" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z29),COUNTIF(Feiertage,DATE(Planungsjahr,6,Z29))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="88" priority="213" stopIfTrue="1">
+    <cfRule type="expression" dxfId="88" priority="713" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z29),WEEKDAY(DATE(Planungsjahr,6,Z29),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z45:AT45 Z47:AT47 Z49:AT49 Z51:AT51 Z53:AT53 Z55:AT55">
-    <cfRule type="expression" dxfId="87" priority="221" stopIfTrue="1">
+    <cfRule type="expression" dxfId="87" priority="721" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z45),WEEKDAY(DATE(Planungsjahr,10,Z45),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="87" priority="220" stopIfTrue="1">
+    <cfRule type="expression" dxfId="87" priority="720" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z45),COUNTIF(Feiertage,DATE(Planungsjahr,10,Z45))&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AE7 AX7">
-    <cfRule type="expression" dxfId="85" priority="201">
-      <formula>LEFT(AE7,1)="⚠"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AP62:AP81">
-    <cfRule type="expression" dxfId="84" priority="232">
+    <cfRule type="expression" dxfId="84" priority="732">
       <formula>AND(ISNUMBER(AP62),YEAR(AP62)&lt;&gt;Planungsjahr)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW13:BQ13 AW15:BQ15 AW17:BQ17 AW19:BQ19 AW21:BQ21 AW23:BQ23">
-    <cfRule type="expression" dxfId="83" priority="207" stopIfTrue="1">
+    <cfRule type="expression" dxfId="83" priority="707" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW13),WEEKDAY(DATE(Planungsjahr,3,AW13),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="206" stopIfTrue="1">
+    <cfRule type="expression" dxfId="83" priority="706" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW13),COUNTIF(Feiertage,DATE(Planungsjahr,3,AW13))&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW29:BQ29 AW31:BQ31 AW33:BQ33 AW35:BQ35 AW37:BQ37 AW39:BQ39">
-    <cfRule type="expression" dxfId="81" priority="215" stopIfTrue="1">
+    <cfRule type="expression" dxfId="81" priority="715" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW29),WEEKDAY(DATE(Planungsjahr,7,AW29),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="214" stopIfTrue="1">
+    <cfRule type="expression" dxfId="81" priority="714" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW29),COUNTIF(Feiertage,DATE(Planungsjahr,7,AW29))&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW45:BQ45 AW47:BQ47 AW49:BQ49 AW51:BQ51 AW53:BQ53 AW55:BQ55">
-    <cfRule type="expression" dxfId="78" priority="222" stopIfTrue="1">
+    <cfRule type="expression" dxfId="78" priority="722" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW45),COUNTIF(Feiertage,DATE(Planungsjahr,11,AW45))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="223" stopIfTrue="1">
+    <cfRule type="expression" dxfId="78" priority="723" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW45),WEEKDAY(DATE(Planungsjahr,11,AW45),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BD62:BD81">
-    <cfRule type="expression" dxfId="77" priority="233">
+    <cfRule type="expression" dxfId="77" priority="733">
       <formula>AND(ISNUMBER(BD62),YEAR(BD62)&lt;&gt;Planungsjahr)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="76" priority="234">
+    <cfRule type="expression" dxfId="76" priority="734">
       <formula>AND(ISNUMBER(BD62),ISNUMBER(SEARCH("prüfen",$BU62)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BD63:BD81">
-    <cfRule type="expression" dxfId="75" priority="235">
+    <cfRule type="expression" dxfId="75" priority="735">
       <formula>AND(ISNUMBER(BD63),ISNUMBER(BD62),BD63&lt;BD62)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT13:CN13 BT15:CN15 BT17:CN17 BT19:CN19 BT21:CN21 BT23:CN23">
-    <cfRule type="expression" dxfId="74" priority="209" stopIfTrue="1">
+    <cfRule type="expression" dxfId="74" priority="709" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT13),WEEKDAY(DATE(Planungsjahr,4,BT13),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="208" stopIfTrue="1">
+    <cfRule type="expression" dxfId="74" priority="708" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT13),COUNTIF(Feiertage,DATE(Planungsjahr,4,BT13))&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT29:CN29 BT31:CN31 BT33:CN33 BT35:CN35 BT37:CN37 BT39:CN39">
-    <cfRule type="expression" dxfId="71" priority="216" stopIfTrue="1">
+    <cfRule type="expression" dxfId="71" priority="716" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT29),COUNTIF(Feiertage,DATE(Planungsjahr,8,BT29))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="217" stopIfTrue="1">
+    <cfRule type="expression" dxfId="71" priority="717" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT29),WEEKDAY(DATE(Planungsjahr,8,BT29),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT45:CN45 BT47:CN47 BT49:CN49 BT51:CN51 BT53:CN53 BT55:CN55">
-    <cfRule type="expression" dxfId="69" priority="224" stopIfTrue="1">
+    <cfRule type="expression" dxfId="69" priority="724" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT45),COUNTIF(Feiertage,DATE(Planungsjahr,12,BT45))&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="69" priority="225" stopIfTrue="1">
+    <cfRule type="expression" dxfId="69" priority="725" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT45),WEEKDAY(DATE(Planungsjahr,12,BT45),2)&gt;5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Art der Bitte" prompt="Bitte auswählen: aktiv, passiv oder nein" sqref="BM62:BM81" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"aktiv,passiv,nein"</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="PAL" error="Bitte ein Datum eingeben." promptTitle="PAL" prompt="Geplanter Eingang bei der Zielgruppe (Briefkasten-Termin), z. B. 26.11.2027" sqref="BD62:BD81" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vorlauf Selektion" error="Bitte eine ganze Zahl ≥ 0 eingeben." promptTitle="Vorlauf Selektion" prompt="Tage vor PAL. Vorbelegt mit dem Standardwert oben – bei Bedarf einfach mit eigener Zahl überschreiben." sqref="AI62:AI81" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vorlauf Selektion" error="Bitte eine ganze Zahl ≥ 0 eingeben." promptTitle="Vorlauf Selektion" prompt="Tage vor PAL. Sommer- und Weihnachtsmailing: automatisch aus dem Gantt (Blatt 2/3), bitte nicht überschreiben. Alle anderen Maßnahmen: hier eintragen." sqref="AI62:AI81" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vorlauf Inhalt" error="Bitte eine ganze Zahl ≥ 0 eingeben." promptTitle="Vorlauf Inhalt" prompt="Tage vor PAL. Vorbelegt mit dem Standardwert oben – bei Bedarf einfach mit eigener Zahl überschreiben." sqref="AW62:AW81" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vorlauf Inhalt" error="Bitte eine ganze Zahl ≥ 0 eingeben." promptTitle="Vorlauf Inhalt" prompt="Tage vor PAL. Sommer- und Weihnachtsmailing: automatisch aus dem Gantt (Blatt 2/3), bitte nicht überschreiben. Alle anderen Maßnahmen: hier eintragen." sqref="AW62:AW81" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Auflage" error="Bitte eine ganze Zahl eingeben." promptTitle="Auflage" prompt="Geplante Auflage (optional, Hinweisfeld)" sqref="V62:V81" xr:uid="{00000000-0002-0000-0000-000004000000}">
@@ -19968,12 +19929,6 @@
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Planungsjahr" error="Bitte ein Jahr zwischen 2000 und 2100 eingeben." promptTitle="Planungsjahr" prompt="Jahr ändern: Kalender und Feiertage passen sich automatisch an." sqref="W4" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>2000</formula1>
       <formula2>2100</formula2>
-    </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vorlauf Selektion" error="Bitte eine ganze Zahl ≥ 0 eingeben." promptTitle="Vorlauf Selektion" prompt="Gantt: Selektion einleiten 2 + Freigabe 5 + Selektion erstellen 52 + Produktion &amp; Versand 17 = 76 Tage. Gilt für alle Zeilen ohne eigenen Wert." sqref="W5" xr:uid="{00000000-0002-0000-0000-000006000000}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Vorlauf Inhalt" error="Bitte eine ganze Zahl ≥ 0 eingeben." promptTitle="Vorlauf Inhalt" prompt="Gantt: Thema 1 + Texte 7 + Gestaltung 14 + Korrektur 5 + Freigaben 14 + Produktion &amp; Versand 17 = 58 Tage. Gilt für alle Zeilen ohne eigenen Wert." sqref="W6" xr:uid="{00000000-0002-0000-0000-000007000000}">
-      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -19986,7 +19941,7 @@
     <brk id="58" max="16383" man="1"/>
   </rowBreaks>
   <ignoredErrors>
-    <ignoredError sqref="B11:CN57" evalError="1" twoDigitTextYear="1" numberStoredAsText="1" formula="1" formulaRange="1" unlockedFormula="1" emptyCellReference="1"/>
+    <ignoredError sqref="B11:CO57" evalError="1" twoDigitTextYear="1" numberStoredAsText="1" formula="1" formulaRange="1" unlockedFormula="1" emptyCellReference="1"/>
   </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -20908,14 +20863,15 @@
       </c>
       <c r="E11" s="57"/>
       <c r="F11" s="70">
-        <f>INDEX(JP_StartSel,MATCH($E$4,JP_Massnahme,0))</f>
+        <f>Plan_Sommer[[#This Row],[Ende]]-Plan_Sommer[[#This Row],[Dauer
+in Tage]]</f>
         <v>46481</v>
       </c>
       <c r="G11" s="71">
         <v>2</v>
       </c>
       <c r="H11" s="72">
-        <f>F11+G11</f>
+        <f>F13</f>
         <v>46483</v>
       </c>
       <c r="I11" s="44" t="str">
@@ -21231,14 +21187,15 @@
       <c r="D13" s="56"/>
       <c r="E13" s="57"/>
       <c r="F13" s="70">
-        <f>H11</f>
+        <f>Plan_Sommer[[#This Row],[Ende]]-Plan_Sommer[[#This Row],[Dauer
+in Tage]]</f>
         <v>46483</v>
       </c>
       <c r="G13" s="71">
         <v>5</v>
       </c>
       <c r="H13" s="72">
-        <f>F13+G13</f>
+        <f>F14</f>
         <v>46488</v>
       </c>
       <c r="I13" s="44" t="str">
@@ -21478,11 +21435,11 @@
       </c>
       <c r="E14" s="57"/>
       <c r="F14" s="70">
-        <f>H13</f>
+        <f>Plan_Sommer[[#This Row],[Ende]]-Plan_Sommer[[#This Row],[Dauer
+in Tage]]</f>
         <v>46488</v>
       </c>
       <c r="G14" s="71">
-        <f>H14-F14</f>
         <v>52</v>
       </c>
       <c r="H14" s="72">
@@ -22205,11 +22162,11 @@
       <c r="D17" s="63"/>
       <c r="E17" s="57"/>
       <c r="F17" s="70">
-        <f>INDEX(JP_StartInhalt,MATCH($E$4,JP_Massnahme,0))</f>
+        <f>Plan_Sommer[[#This Row],[Ende]]-Plan_Sommer[[#This Row],[Dauer
+in Tage]]</f>
         <v>46499</v>
       </c>
       <c r="G17" s="71">
-        <f>H17-F17</f>
         <v>1</v>
       </c>
       <c r="H17" s="72">
@@ -29285,11 +29242,6 @@
       <formula>AND(TODAY()&gt;=F$7,TODAY()&lt;G$7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G14 G17">
-    <cfRule type="cellIs" dxfId="47" priority="3000" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="I6:AM6">
     <cfRule type="expression" dxfId="46" priority="54">
       <formula>I$7&lt;=EOMONTH($I$7,0)</formula>
@@ -29342,7 +29294,7 @@
       <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
+  <dataValidations count="10">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10" xr:uid="{E87210D7-3045-41D8-B549-D8254C353C87}">
       <formula1>"Ziel,Meilenstein,Im Plan, Geringes Risiko, Mittleres Risiko, Hohes Risiko"</formula1>
     </dataValidation>
@@ -29357,12 +29309,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C11:C45" xr:uid="{2B59BEAD-9C8D-422A-A3A2-A5C66751BF48}">
       <formula1>$C$5:$H$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Verknüpfung" prompt="Name der Maßnahme auf Blatt „Jahresplanung“. Von hier kommen PAL, Start Selektion und Start inhaltliche Arbeit." sqref="E4" xr:uid="{00000000-0002-0000-0100-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Verknüpfung" prompt="Name der Maßnahme auf Blatt „Jahresplanung“. Von hier kommt der PAL (Briefkasten-Datum). Der Vorlauf wird aus diesem Gantt nach Blatt 1 übertragen." sqref="E4" xr:uid="{00000000-0002-0000-0100-000008000000}">
       <formula1>JP_Massnahme</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Briefkasten-Datum (PAL)" prompt="Wird aus Blatt „Jahresplanung“ übernommen – bitte dort ändern." sqref="C4" xr:uid="{00000000-0002-0000-0100-000009000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Start Selektion" prompt="Kommt aus Blatt „Jahresplanung“ (PAL − Vorlauf Selektion). „Selektion erstellen“ füllt die Zeit bis zur Übergabe an den Lettershop." sqref="F11" xr:uid="{00000000-0002-0000-0100-00000A000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Start inhaltliche Arbeit" prompt="Kommt aus Blatt „Jahresplanung“ (PAL − Vorlauf Inhalt). „Thema definieren“ dauert bis zum Beginn der Texterstellung." sqref="F17" xr:uid="{00000000-0002-0000-0100-00000B000000}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -30381,14 +30331,15 @@
       </c>
       <c r="E11" s="57"/>
       <c r="F11" s="70">
-        <f>INDEX(JP_StartSel,MATCH($E$4,JP_Massnahme,0))</f>
+        <f>Plan_Weihnachten[[#This Row],[Ende]]-Plan_Weihnachten[[#This Row],[Dauer
+in Tage]]</f>
         <v>46641</v>
       </c>
       <c r="G11" s="71">
         <v>2</v>
       </c>
       <c r="H11" s="72">
-        <f>F11+G11</f>
+        <f>F13</f>
         <v>46643</v>
       </c>
       <c r="I11" s="44" t="str">
@@ -30704,14 +30655,15 @@
       <c r="D13" s="56"/>
       <c r="E13" s="57"/>
       <c r="F13" s="70">
-        <f>H11</f>
+        <f>Plan_Weihnachten[[#This Row],[Ende]]-Plan_Weihnachten[[#This Row],[Dauer
+in Tage]]</f>
         <v>46643</v>
       </c>
       <c r="G13" s="71">
         <v>5</v>
       </c>
       <c r="H13" s="72">
-        <f>F13+G13</f>
+        <f>F14</f>
         <v>46648</v>
       </c>
       <c r="I13" s="44" t="str">
@@ -30951,11 +30903,11 @@
       </c>
       <c r="E14" s="57"/>
       <c r="F14" s="70">
-        <f>H13</f>
+        <f>Plan_Weihnachten[[#This Row],[Ende]]-Plan_Weihnachten[[#This Row],[Dauer
+in Tage]]</f>
         <v>46648</v>
       </c>
       <c r="G14" s="71">
-        <f>H14-F14</f>
         <v>52</v>
       </c>
       <c r="H14" s="72">
@@ -31678,11 +31630,11 @@
       <c r="D17" s="63"/>
       <c r="E17" s="57"/>
       <c r="F17" s="70">
-        <f>INDEX(JP_StartInhalt,MATCH($E$4,JP_Massnahme,0))</f>
+        <f>Plan_Weihnachten[[#This Row],[Ende]]-Plan_Weihnachten[[#This Row],[Dauer
+in Tage]]</f>
         <v>46659</v>
       </c>
       <c r="G17" s="71">
-        <f>H17-F17</f>
         <v>1</v>
       </c>
       <c r="H17" s="72">
@@ -38758,11 +38710,6 @@
       <formula>AND(TODAY()&gt;=F$7,TODAY()&lt;G$7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G14 G17">
-    <cfRule type="cellIs" dxfId="13" priority="3000" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="I6:AM6">
     <cfRule type="expression" dxfId="12" priority="54">
       <formula>I$7&lt;=EOMONTH($I$7,0)</formula>
@@ -38815,7 +38762,7 @@
       <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
+  <dataValidations count="10">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10" xr:uid="{AE36670D-A762-476F-A998-26F2E53DA15E}">
       <formula1>"Ziel,Meilenstein,Im Plan, Geringes Risiko, Mittleres Risiko, Hohes Risiko"</formula1>
     </dataValidation>
@@ -38830,12 +38777,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C11:C45" xr:uid="{1FA86119-1C0F-4FE6-BDF6-8944579FCF85}">
       <formula1>$C$5:$H$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Verknüpfung" prompt="Name der Maßnahme auf Blatt „Jahresplanung“. Von hier kommen PAL, Start Selektion und Start inhaltliche Arbeit." sqref="E4" xr:uid="{00000000-0002-0000-0200-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Verknüpfung" prompt="Name der Maßnahme auf Blatt „Jahresplanung“. Von hier kommt der PAL (Briefkasten-Datum). Der Vorlauf wird aus diesem Gantt nach Blatt 1 übertragen." sqref="E4" xr:uid="{00000000-0002-0000-0200-000008000000}">
       <formula1>JP_Massnahme</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Briefkasten-Datum (PAL)" prompt="Wird aus Blatt „Jahresplanung“ übernommen – bitte dort ändern." sqref="C4" xr:uid="{00000000-0002-0000-0200-000009000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Start Selektion" prompt="Kommt aus Blatt „Jahresplanung“ (PAL − Vorlauf Selektion). „Selektion erstellen“ füllt die Zeit bis zur Übergabe an den Lettershop." sqref="F11" xr:uid="{00000000-0002-0000-0200-00000A000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Start inhaltliche Arbeit" prompt="Kommt aus Blatt „Jahresplanung“ (PAL − Vorlauf Inhalt). „Thema definieren“ dauert bis zum Beginn der Texterstellung." sqref="F17" xr:uid="{00000000-0002-0000-0200-00000B000000}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Jahresplanung: Kontrollkästchen in einzelnen Zellen, Feiertage schraffiert
- Kontrollkästchen S/I/P in nicht verbundene Einzelzellen (S, T, U)
  verlegt, da Excel sie in verbundenen Zellen nicht zeichnet
- Feiertage im Kalender und in der Legende: fette Schrift, grau
  schraffierter Hintergrund (Wochenenden bleiben flächig grau)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Efpubc9TCkNCWzy5pGdKJy
</commit_message>
<xml_diff>
--- a/excel/260924_Jahresplanung_Aussenkommunikation_2027_MA.xlsx
+++ b/excel/260924_Jahresplanung_Aussenkommunikation_2027_MA.xlsx
@@ -24,9 +24,9 @@
     <definedName name="JP_Auflage">Jahresplanung!$V$62:$V$81</definedName>
     <definedName name="JP_Massnahme">Jahresplanung!$B$62:$B$81</definedName>
     <definedName name="JP_PAL">Jahresplanung!$BD$62:$BD$81</definedName>
-    <definedName name="JP_ShowInhalt">Jahresplanung!$R$62:$R$81</definedName>
-    <definedName name="JP_ShowPAL">Jahresplanung!$T$62:$T$81</definedName>
-    <definedName name="JP_ShowSel">Jahresplanung!$P$62:$P$81</definedName>
+    <definedName name="JP_ShowInhalt">Jahresplanung!$T$62:$T$81</definedName>
+    <definedName name="JP_ShowPAL">Jahresplanung!$U$62:$U$81</definedName>
+    <definedName name="JP_ShowSel">Jahresplanung!$S$62:$S$81</definedName>
     <definedName name="JP_StartInhalt">Jahresplanung!$AP$62:$AP$81</definedName>
     <definedName name="JP_StartSel">Jahresplanung!$Z$62:$Z$81</definedName>
     <definedName name="JP_VorlaufInhalt">Jahresplanung!$AW$62:$AW$81</definedName>
@@ -618,7 +618,7 @@
     <numFmt numFmtId="169" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="170" formatCode="[$-407]dddd"/>
   </numFmts>
-  <fonts count="70" x14ac:knownFonts="1">
+  <fonts count="74" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1136,8 +1136,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF548235"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFE30714"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF404040"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1255,6 +1284,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="lightUp">
+        <fgColor rgb="FFA6A6A6"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -1927,7 +1962,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="205">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2524,6 +2559,33 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="70" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="21" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Akzent3" xfId="11" builtinId="37"/>
@@ -2539,7 +2601,7 @@
     <cellStyle name="Überschrift 3" xfId="8" builtinId="18" customBuiltin="1"/>
     <cellStyle name="zAusgeblText" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="142">
+  <dxfs count="144">
     <dxf>
       <font>
         <i/>
@@ -4048,6 +4110,27 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF404040"/>
+      </font>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor rgb="FFA6A6A6"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="200" formatCode=";;;"/>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor rgb="FFA6A6A6"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Gantt-Tabellenformat" pivot="0" count="4" xr9:uid="{4904D139-63E4-4221-B7C9-C6C5B7A50FAF}">
@@ -5160,10 +5243,10 @@
       <c r="BZ7" s="121"/>
       <c r="CA7" s="121"/>
       <c r="CB7" s="121"/>
-      <c r="CD7" s="122" t="s">
+      <c r="CD7" s="204" t="s">
         <v>68</v>
       </c>
-      <c r="CE7" s="122"/>
+      <c r="CE7" s="204"/>
       <c r="CF7" s="121" t="s">
         <v>70</v>
       </c>
@@ -15970,18 +16053,18 @@
       <c r="M61" s="127"/>
       <c r="N61" s="127"/>
       <c r="O61" s="127"/>
-      <c r="P61" s="129" t="s">
+      <c r="P61" s="127"/>
+      <c r="Q61" s="127"/>
+      <c r="R61" s="127"/>
+      <c r="S61" s="129" t="s">
         <v>154</v>
       </c>
-      <c r="Q61" s="129"/>
-      <c r="R61" s="131" t="s">
+      <c r="T61" s="131" t="s">
         <v>155</v>
       </c>
-      <c r="S61" s="131"/>
-      <c r="T61" s="133" t="s">
+      <c r="U61" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="U61" s="133"/>
       <c r="V61" s="128" t="s">
         <v>82</v>
       </c>
@@ -16087,18 +16170,18 @@
       <c r="M62" s="134"/>
       <c r="N62" s="134"/>
       <c r="O62" s="134"/>
-      <c r="P62" s="198" t="b">
+      <c r="P62" s="134"/>
+      <c r="Q62" s="134"/>
+      <c r="R62" s="134"/>
+      <c r="S62" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q62" s="139"/>
-      <c r="R62" s="199" t="b">
+      <c r="T62" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S62" s="139"/>
-      <c r="T62" s="200" t="b">
+      <c r="U62" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U62" s="139"/>
       <c r="V62" s="135"/>
       <c r="W62" s="135"/>
       <c r="X62" s="135"/>
@@ -16202,18 +16285,18 @@
       <c r="M63" s="134"/>
       <c r="N63" s="134"/>
       <c r="O63" s="134"/>
-      <c r="P63" s="198" t="b">
+      <c r="P63" s="134"/>
+      <c r="Q63" s="134"/>
+      <c r="R63" s="134"/>
+      <c r="S63" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q63" s="139"/>
-      <c r="R63" s="199" t="b">
+      <c r="T63" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S63" s="139"/>
-      <c r="T63" s="200" t="b">
+      <c r="U63" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U63" s="139"/>
       <c r="V63" s="135"/>
       <c r="W63" s="135"/>
       <c r="X63" s="135"/>
@@ -16317,18 +16400,18 @@
       <c r="M64" s="134"/>
       <c r="N64" s="134"/>
       <c r="O64" s="134"/>
-      <c r="P64" s="198" t="b">
+      <c r="P64" s="134"/>
+      <c r="Q64" s="134"/>
+      <c r="R64" s="134"/>
+      <c r="S64" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q64" s="139"/>
-      <c r="R64" s="199" t="b">
+      <c r="T64" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S64" s="139"/>
-      <c r="T64" s="200" t="b">
+      <c r="U64" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U64" s="139"/>
       <c r="V64" s="135"/>
       <c r="W64" s="135"/>
       <c r="X64" s="135"/>
@@ -16432,18 +16515,18 @@
       <c r="M65" s="134"/>
       <c r="N65" s="134"/>
       <c r="O65" s="134"/>
-      <c r="P65" s="198" t="b">
+      <c r="P65" s="134"/>
+      <c r="Q65" s="134"/>
+      <c r="R65" s="134"/>
+      <c r="S65" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q65" s="139"/>
-      <c r="R65" s="199" t="b">
+      <c r="T65" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S65" s="139"/>
-      <c r="T65" s="200" t="b">
+      <c r="U65" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U65" s="139"/>
       <c r="V65" s="135"/>
       <c r="W65" s="135"/>
       <c r="X65" s="135"/>
@@ -16551,18 +16634,18 @@
       <c r="M66" s="134"/>
       <c r="N66" s="134"/>
       <c r="O66" s="134"/>
-      <c r="P66" s="198" t="b">
+      <c r="P66" s="134"/>
+      <c r="Q66" s="134"/>
+      <c r="R66" s="134"/>
+      <c r="S66" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q66" s="139"/>
-      <c r="R66" s="199" t="b">
+      <c r="T66" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S66" s="139"/>
-      <c r="T66" s="200" t="b">
+      <c r="U66" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U66" s="139"/>
       <c r="V66" s="135"/>
       <c r="W66" s="135"/>
       <c r="X66" s="135"/>
@@ -16666,18 +16749,18 @@
       <c r="M67" s="134"/>
       <c r="N67" s="134"/>
       <c r="O67" s="134"/>
-      <c r="P67" s="198" t="b">
+      <c r="P67" s="134"/>
+      <c r="Q67" s="134"/>
+      <c r="R67" s="134"/>
+      <c r="S67" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q67" s="139"/>
-      <c r="R67" s="199" t="b">
+      <c r="T67" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S67" s="139"/>
-      <c r="T67" s="200" t="b">
+      <c r="U67" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U67" s="139"/>
       <c r="V67" s="135"/>
       <c r="W67" s="135"/>
       <c r="X67" s="135"/>
@@ -16781,18 +16864,18 @@
       <c r="M68" s="134"/>
       <c r="N68" s="134"/>
       <c r="O68" s="134"/>
-      <c r="P68" s="198" t="b">
+      <c r="P68" s="134"/>
+      <c r="Q68" s="134"/>
+      <c r="R68" s="134"/>
+      <c r="S68" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q68" s="139"/>
-      <c r="R68" s="199" t="b">
+      <c r="T68" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S68" s="139"/>
-      <c r="T68" s="200" t="b">
+      <c r="U68" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U68" s="139"/>
       <c r="V68" s="135"/>
       <c r="W68" s="135"/>
       <c r="X68" s="135"/>
@@ -16898,18 +16981,18 @@
       <c r="M69" s="134"/>
       <c r="N69" s="134"/>
       <c r="O69" s="134"/>
-      <c r="P69" s="198" t="b">
+      <c r="P69" s="134"/>
+      <c r="Q69" s="134"/>
+      <c r="R69" s="134"/>
+      <c r="S69" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q69" s="139"/>
-      <c r="R69" s="199" t="b">
+      <c r="T69" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S69" s="139"/>
-      <c r="T69" s="200" t="b">
+      <c r="U69" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U69" s="139"/>
       <c r="V69" s="135"/>
       <c r="W69" s="135"/>
       <c r="X69" s="135"/>
@@ -17013,18 +17096,18 @@
       <c r="M70" s="134"/>
       <c r="N70" s="134"/>
       <c r="O70" s="134"/>
-      <c r="P70" s="198" t="b">
+      <c r="P70" s="134"/>
+      <c r="Q70" s="134"/>
+      <c r="R70" s="134"/>
+      <c r="S70" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q70" s="139"/>
-      <c r="R70" s="199" t="b">
+      <c r="T70" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S70" s="139"/>
-      <c r="T70" s="200" t="b">
+      <c r="U70" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U70" s="139"/>
       <c r="V70" s="135"/>
       <c r="W70" s="135"/>
       <c r="X70" s="135"/>
@@ -17132,18 +17215,18 @@
       <c r="M71" s="134"/>
       <c r="N71" s="134"/>
       <c r="O71" s="134"/>
-      <c r="P71" s="198" t="b">
+      <c r="P71" s="134"/>
+      <c r="Q71" s="134"/>
+      <c r="R71" s="134"/>
+      <c r="S71" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q71" s="139"/>
-      <c r="R71" s="199" t="b">
+      <c r="T71" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S71" s="139"/>
-      <c r="T71" s="200" t="b">
+      <c r="U71" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U71" s="139"/>
       <c r="V71" s="135"/>
       <c r="W71" s="135"/>
       <c r="X71" s="135"/>
@@ -17245,18 +17328,18 @@
       <c r="M72" s="134"/>
       <c r="N72" s="134"/>
       <c r="O72" s="134"/>
-      <c r="P72" s="198" t="b">
+      <c r="P72" s="134"/>
+      <c r="Q72" s="134"/>
+      <c r="R72" s="134"/>
+      <c r="S72" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q72" s="139"/>
-      <c r="R72" s="199" t="b">
+      <c r="T72" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S72" s="139"/>
-      <c r="T72" s="200" t="b">
+      <c r="U72" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U72" s="139"/>
       <c r="V72" s="135"/>
       <c r="W72" s="135"/>
       <c r="X72" s="135"/>
@@ -17350,18 +17433,18 @@
       <c r="M73" s="134"/>
       <c r="N73" s="134"/>
       <c r="O73" s="134"/>
-      <c r="P73" s="198" t="b">
+      <c r="P73" s="134"/>
+      <c r="Q73" s="134"/>
+      <c r="R73" s="134"/>
+      <c r="S73" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q73" s="139"/>
-      <c r="R73" s="199" t="b">
+      <c r="T73" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S73" s="139"/>
-      <c r="T73" s="200" t="b">
+      <c r="U73" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U73" s="139"/>
       <c r="V73" s="135"/>
       <c r="W73" s="135"/>
       <c r="X73" s="135"/>
@@ -17455,18 +17538,18 @@
       <c r="M74" s="134"/>
       <c r="N74" s="134"/>
       <c r="O74" s="134"/>
-      <c r="P74" s="198" t="b">
+      <c r="P74" s="134"/>
+      <c r="Q74" s="134"/>
+      <c r="R74" s="134"/>
+      <c r="S74" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q74" s="139"/>
-      <c r="R74" s="199" t="b">
+      <c r="T74" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S74" s="139"/>
-      <c r="T74" s="200" t="b">
+      <c r="U74" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U74" s="139"/>
       <c r="V74" s="135"/>
       <c r="W74" s="135"/>
       <c r="X74" s="135"/>
@@ -17560,18 +17643,18 @@
       <c r="M75" s="134"/>
       <c r="N75" s="134"/>
       <c r="O75" s="134"/>
-      <c r="P75" s="198" t="b">
+      <c r="P75" s="134"/>
+      <c r="Q75" s="134"/>
+      <c r="R75" s="134"/>
+      <c r="S75" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q75" s="139"/>
-      <c r="R75" s="199" t="b">
+      <c r="T75" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S75" s="139"/>
-      <c r="T75" s="200" t="b">
+      <c r="U75" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U75" s="139"/>
       <c r="V75" s="135"/>
       <c r="W75" s="135"/>
       <c r="X75" s="135"/>
@@ -17665,18 +17748,18 @@
       <c r="M76" s="134"/>
       <c r="N76" s="134"/>
       <c r="O76" s="134"/>
-      <c r="P76" s="198" t="b">
+      <c r="P76" s="134"/>
+      <c r="Q76" s="134"/>
+      <c r="R76" s="134"/>
+      <c r="S76" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q76" s="139"/>
-      <c r="R76" s="199" t="b">
+      <c r="T76" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S76" s="139"/>
-      <c r="T76" s="200" t="b">
+      <c r="U76" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U76" s="139"/>
       <c r="V76" s="135"/>
       <c r="W76" s="135"/>
       <c r="X76" s="135"/>
@@ -17770,18 +17853,18 @@
       <c r="M77" s="134"/>
       <c r="N77" s="134"/>
       <c r="O77" s="134"/>
-      <c r="P77" s="198" t="b">
+      <c r="P77" s="134"/>
+      <c r="Q77" s="134"/>
+      <c r="R77" s="134"/>
+      <c r="S77" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q77" s="139"/>
-      <c r="R77" s="199" t="b">
+      <c r="T77" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S77" s="139"/>
-      <c r="T77" s="200" t="b">
+      <c r="U77" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U77" s="139"/>
       <c r="V77" s="135"/>
       <c r="W77" s="135"/>
       <c r="X77" s="135"/>
@@ -17875,18 +17958,18 @@
       <c r="M78" s="134"/>
       <c r="N78" s="134"/>
       <c r="O78" s="134"/>
-      <c r="P78" s="198" t="b">
+      <c r="P78" s="134"/>
+      <c r="Q78" s="134"/>
+      <c r="R78" s="134"/>
+      <c r="S78" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q78" s="139"/>
-      <c r="R78" s="199" t="b">
+      <c r="T78" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S78" s="139"/>
-      <c r="T78" s="200" t="b">
+      <c r="U78" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U78" s="139"/>
       <c r="V78" s="135"/>
       <c r="W78" s="135"/>
       <c r="X78" s="135"/>
@@ -17980,18 +18063,18 @@
       <c r="M79" s="134"/>
       <c r="N79" s="134"/>
       <c r="O79" s="134"/>
-      <c r="P79" s="198" t="b">
+      <c r="P79" s="134"/>
+      <c r="Q79" s="134"/>
+      <c r="R79" s="134"/>
+      <c r="S79" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q79" s="139"/>
-      <c r="R79" s="199" t="b">
+      <c r="T79" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S79" s="139"/>
-      <c r="T79" s="200" t="b">
+      <c r="U79" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U79" s="139"/>
       <c r="V79" s="135"/>
       <c r="W79" s="135"/>
       <c r="X79" s="135"/>
@@ -18085,18 +18168,18 @@
       <c r="M80" s="134"/>
       <c r="N80" s="134"/>
       <c r="O80" s="134"/>
-      <c r="P80" s="198" t="b">
+      <c r="P80" s="134"/>
+      <c r="Q80" s="134"/>
+      <c r="R80" s="134"/>
+      <c r="S80" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q80" s="139"/>
-      <c r="R80" s="199" t="b">
+      <c r="T80" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S80" s="139"/>
-      <c r="T80" s="200" t="b">
+      <c r="U80" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U80" s="139"/>
       <c r="V80" s="135"/>
       <c r="W80" s="135"/>
       <c r="X80" s="135"/>
@@ -18190,18 +18273,18 @@
       <c r="M81" s="134"/>
       <c r="N81" s="134"/>
       <c r="O81" s="134"/>
-      <c r="P81" s="198" t="b">
+      <c r="P81" s="134"/>
+      <c r="Q81" s="134"/>
+      <c r="R81" s="134"/>
+      <c r="S81" s="201" t="b">
         <v>1</v>
       </c>
-      <c r="Q81" s="139"/>
-      <c r="R81" s="199" t="b">
+      <c r="T81" s="202" t="b">
         <v>1</v>
       </c>
-      <c r="S81" s="139"/>
-      <c r="T81" s="200" t="b">
+      <c r="U81" s="203" t="b">
         <v>1</v>
       </c>
-      <c r="U81" s="139"/>
       <c r="V81" s="135"/>
       <c r="W81" s="135"/>
       <c r="X81" s="135"/>
@@ -18761,17 +18844,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="803">
+  <mergeCells count="740">
     <mergeCell ref="B83:CN83"/>
     <mergeCell ref="B84:CN84"/>
     <mergeCell ref="B85:CN85"/>
     <mergeCell ref="B86:CN86"/>
     <mergeCell ref="B87:CN87"/>
     <mergeCell ref="B88:CN88"/>
-    <mergeCell ref="B81:O81"/>
-    <mergeCell ref="P81:Q81"/>
-    <mergeCell ref="R81:S81"/>
-    <mergeCell ref="T81:U81"/>
     <mergeCell ref="V81:Y81"/>
     <mergeCell ref="Z81:AH81"/>
     <mergeCell ref="AI81:AO81"/>
@@ -18780,10 +18859,6 @@
     <mergeCell ref="BD81:BL81"/>
     <mergeCell ref="BM81:BT81"/>
     <mergeCell ref="BU81:CN81"/>
-    <mergeCell ref="B80:O80"/>
-    <mergeCell ref="P80:Q80"/>
-    <mergeCell ref="R80:S80"/>
-    <mergeCell ref="T80:U80"/>
     <mergeCell ref="V80:Y80"/>
     <mergeCell ref="Z80:AH80"/>
     <mergeCell ref="AI80:AO80"/>
@@ -18792,10 +18867,6 @@
     <mergeCell ref="BD80:BL80"/>
     <mergeCell ref="BM80:BT80"/>
     <mergeCell ref="BU80:CN80"/>
-    <mergeCell ref="B79:O79"/>
-    <mergeCell ref="P79:Q79"/>
-    <mergeCell ref="R79:S79"/>
-    <mergeCell ref="T79:U79"/>
     <mergeCell ref="V79:Y79"/>
     <mergeCell ref="Z79:AH79"/>
     <mergeCell ref="AI79:AO79"/>
@@ -18804,10 +18875,6 @@
     <mergeCell ref="BD79:BL79"/>
     <mergeCell ref="BM79:BT79"/>
     <mergeCell ref="BU79:CN79"/>
-    <mergeCell ref="B78:O78"/>
-    <mergeCell ref="P78:Q78"/>
-    <mergeCell ref="R78:S78"/>
-    <mergeCell ref="T78:U78"/>
     <mergeCell ref="V78:Y78"/>
     <mergeCell ref="Z78:AH78"/>
     <mergeCell ref="AI78:AO78"/>
@@ -18816,10 +18883,6 @@
     <mergeCell ref="BD78:BL78"/>
     <mergeCell ref="BM78:BT78"/>
     <mergeCell ref="BU78:CN78"/>
-    <mergeCell ref="B77:O77"/>
-    <mergeCell ref="P77:Q77"/>
-    <mergeCell ref="R77:S77"/>
-    <mergeCell ref="T77:U77"/>
     <mergeCell ref="V77:Y77"/>
     <mergeCell ref="Z77:AH77"/>
     <mergeCell ref="AI77:AO77"/>
@@ -18828,10 +18891,6 @@
     <mergeCell ref="BD77:BL77"/>
     <mergeCell ref="BM77:BT77"/>
     <mergeCell ref="BU77:CN77"/>
-    <mergeCell ref="B76:O76"/>
-    <mergeCell ref="P76:Q76"/>
-    <mergeCell ref="R76:S76"/>
-    <mergeCell ref="T76:U76"/>
     <mergeCell ref="V76:Y76"/>
     <mergeCell ref="Z76:AH76"/>
     <mergeCell ref="AI76:AO76"/>
@@ -18840,10 +18899,6 @@
     <mergeCell ref="BD76:BL76"/>
     <mergeCell ref="BM76:BT76"/>
     <mergeCell ref="BU76:CN76"/>
-    <mergeCell ref="B75:O75"/>
-    <mergeCell ref="P75:Q75"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="T75:U75"/>
     <mergeCell ref="V75:Y75"/>
     <mergeCell ref="Z75:AH75"/>
     <mergeCell ref="AI75:AO75"/>
@@ -18852,10 +18907,6 @@
     <mergeCell ref="BD75:BL75"/>
     <mergeCell ref="BM75:BT75"/>
     <mergeCell ref="BU75:CN75"/>
-    <mergeCell ref="B74:O74"/>
-    <mergeCell ref="P74:Q74"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="T74:U74"/>
     <mergeCell ref="V74:Y74"/>
     <mergeCell ref="Z74:AH74"/>
     <mergeCell ref="AI74:AO74"/>
@@ -18864,10 +18915,6 @@
     <mergeCell ref="BD74:BL74"/>
     <mergeCell ref="BM74:BT74"/>
     <mergeCell ref="BU74:CN74"/>
-    <mergeCell ref="B73:O73"/>
-    <mergeCell ref="P73:Q73"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="T73:U73"/>
     <mergeCell ref="V73:Y73"/>
     <mergeCell ref="Z73:AH73"/>
     <mergeCell ref="AI73:AO73"/>
@@ -18876,10 +18923,6 @@
     <mergeCell ref="BD73:BL73"/>
     <mergeCell ref="BM73:BT73"/>
     <mergeCell ref="BU73:CN73"/>
-    <mergeCell ref="B72:O72"/>
-    <mergeCell ref="P72:Q72"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="T72:U72"/>
     <mergeCell ref="V72:Y72"/>
     <mergeCell ref="Z72:AH72"/>
     <mergeCell ref="AI72:AO72"/>
@@ -18888,10 +18931,6 @@
     <mergeCell ref="BD72:BL72"/>
     <mergeCell ref="BM72:BT72"/>
     <mergeCell ref="BU72:CN72"/>
-    <mergeCell ref="B71:O71"/>
-    <mergeCell ref="P71:Q71"/>
-    <mergeCell ref="R71:S71"/>
-    <mergeCell ref="T71:U71"/>
     <mergeCell ref="V71:Y71"/>
     <mergeCell ref="Z71:AH71"/>
     <mergeCell ref="AI71:AO71"/>
@@ -18900,10 +18939,6 @@
     <mergeCell ref="BD71:BL71"/>
     <mergeCell ref="BM71:BT71"/>
     <mergeCell ref="BU71:CN71"/>
-    <mergeCell ref="B70:O70"/>
-    <mergeCell ref="P70:Q70"/>
-    <mergeCell ref="R70:S70"/>
-    <mergeCell ref="T70:U70"/>
     <mergeCell ref="V70:Y70"/>
     <mergeCell ref="Z70:AH70"/>
     <mergeCell ref="AI70:AO70"/>
@@ -18912,10 +18947,6 @@
     <mergeCell ref="BD70:BL70"/>
     <mergeCell ref="BM70:BT70"/>
     <mergeCell ref="BU70:CN70"/>
-    <mergeCell ref="B69:O69"/>
-    <mergeCell ref="P69:Q69"/>
-    <mergeCell ref="R69:S69"/>
-    <mergeCell ref="T69:U69"/>
     <mergeCell ref="V69:Y69"/>
     <mergeCell ref="Z69:AH69"/>
     <mergeCell ref="AI69:AO69"/>
@@ -18924,10 +18955,6 @@
     <mergeCell ref="BD69:BL69"/>
     <mergeCell ref="BM69:BT69"/>
     <mergeCell ref="BU69:CN69"/>
-    <mergeCell ref="B68:O68"/>
-    <mergeCell ref="P68:Q68"/>
-    <mergeCell ref="R68:S68"/>
-    <mergeCell ref="T68:U68"/>
     <mergeCell ref="V68:Y68"/>
     <mergeCell ref="Z68:AH68"/>
     <mergeCell ref="AI68:AO68"/>
@@ -18936,10 +18963,6 @@
     <mergeCell ref="BD68:BL68"/>
     <mergeCell ref="BM68:BT68"/>
     <mergeCell ref="BU68:CN68"/>
-    <mergeCell ref="B67:O67"/>
-    <mergeCell ref="P67:Q67"/>
-    <mergeCell ref="R67:S67"/>
-    <mergeCell ref="T67:U67"/>
     <mergeCell ref="V67:Y67"/>
     <mergeCell ref="Z67:AH67"/>
     <mergeCell ref="AI67:AO67"/>
@@ -18948,10 +18971,6 @@
     <mergeCell ref="BD67:BL67"/>
     <mergeCell ref="BM67:BT67"/>
     <mergeCell ref="BU67:CN67"/>
-    <mergeCell ref="B66:O66"/>
-    <mergeCell ref="P66:Q66"/>
-    <mergeCell ref="R66:S66"/>
-    <mergeCell ref="T66:U66"/>
     <mergeCell ref="V66:Y66"/>
     <mergeCell ref="Z66:AH66"/>
     <mergeCell ref="AI66:AO66"/>
@@ -18960,10 +18979,6 @@
     <mergeCell ref="BD66:BL66"/>
     <mergeCell ref="BM66:BT66"/>
     <mergeCell ref="BU66:CN66"/>
-    <mergeCell ref="B65:O65"/>
-    <mergeCell ref="P65:Q65"/>
-    <mergeCell ref="R65:S65"/>
-    <mergeCell ref="T65:U65"/>
     <mergeCell ref="V65:Y65"/>
     <mergeCell ref="Z65:AH65"/>
     <mergeCell ref="AI65:AO65"/>
@@ -18972,10 +18987,6 @@
     <mergeCell ref="BD65:BL65"/>
     <mergeCell ref="BM65:BT65"/>
     <mergeCell ref="BU65:CN65"/>
-    <mergeCell ref="B64:O64"/>
-    <mergeCell ref="P64:Q64"/>
-    <mergeCell ref="R64:S64"/>
-    <mergeCell ref="T64:U64"/>
     <mergeCell ref="V64:Y64"/>
     <mergeCell ref="Z64:AH64"/>
     <mergeCell ref="AI64:AO64"/>
@@ -18984,10 +18995,6 @@
     <mergeCell ref="BD64:BL64"/>
     <mergeCell ref="BM64:BT64"/>
     <mergeCell ref="BU64:CN64"/>
-    <mergeCell ref="B63:O63"/>
-    <mergeCell ref="P63:Q63"/>
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="T63:U63"/>
     <mergeCell ref="V63:Y63"/>
     <mergeCell ref="Z63:AH63"/>
     <mergeCell ref="AI63:AO63"/>
@@ -18996,10 +19003,6 @@
     <mergeCell ref="BD63:BL63"/>
     <mergeCell ref="BM63:BT63"/>
     <mergeCell ref="BU63:CN63"/>
-    <mergeCell ref="B62:O62"/>
-    <mergeCell ref="P62:Q62"/>
-    <mergeCell ref="R62:S62"/>
-    <mergeCell ref="T62:U62"/>
     <mergeCell ref="V62:Y62"/>
     <mergeCell ref="Z62:AH62"/>
     <mergeCell ref="AI62:AO62"/>
@@ -19011,10 +19014,6 @@
     <mergeCell ref="BS57:CN57"/>
     <mergeCell ref="B60:AJ60"/>
     <mergeCell ref="AK60:CN60"/>
-    <mergeCell ref="B61:O61"/>
-    <mergeCell ref="P61:Q61"/>
-    <mergeCell ref="R61:S61"/>
-    <mergeCell ref="T61:U61"/>
     <mergeCell ref="V61:Y61"/>
     <mergeCell ref="Z61:AH61"/>
     <mergeCell ref="AI61:AO61"/>
@@ -19565,6 +19564,27 @@
     <mergeCell ref="BV7:CB7"/>
     <mergeCell ref="CD7:CE7"/>
     <mergeCell ref="CF7:CN7"/>
+    <mergeCell ref="B61:R61"/>
+    <mergeCell ref="B62:R62"/>
+    <mergeCell ref="B63:R63"/>
+    <mergeCell ref="B64:R64"/>
+    <mergeCell ref="B65:R65"/>
+    <mergeCell ref="B66:R66"/>
+    <mergeCell ref="B67:R67"/>
+    <mergeCell ref="B68:R68"/>
+    <mergeCell ref="B69:R69"/>
+    <mergeCell ref="B70:R70"/>
+    <mergeCell ref="B71:R71"/>
+    <mergeCell ref="B72:R72"/>
+    <mergeCell ref="B73:R73"/>
+    <mergeCell ref="B74:R74"/>
+    <mergeCell ref="B75:R75"/>
+    <mergeCell ref="B76:R76"/>
+    <mergeCell ref="B77:R77"/>
+    <mergeCell ref="B78:R78"/>
+    <mergeCell ref="B79:R79"/>
+    <mergeCell ref="B80:R80"/>
+    <mergeCell ref="B81:R81"/>
   </mergeCells>
   <conditionalFormatting sqref="C13 F13 I13 L13 O13 R13 U13 C15 F15 I15 L15 O15 R15 U15 C17 F17 I17 L17 O17 R17 U17 C19 F19 I19 L19 O19 R19 U19 C21 F21 I21 L21 O21 R21 U21 C23 F23 I23 L23 O23 R23 U23">
     <cfRule type="expression" dxfId="136" priority="1">
@@ -20047,7 +20067,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:W13 C15:W15 C17:W17 C19:W19 C21:W21 C23:W23">
-    <cfRule type="expression" dxfId="101" priority="702" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="702" stopIfTrue="1">
       <formula>AND(ISNUMBER(C13),COUNTIF(Feiertage,DATE(Planungsjahr,1,C13))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="101" priority="703" stopIfTrue="1">
@@ -20058,7 +20078,7 @@
     <cfRule type="cellIs" dxfId="100" priority="730" stopIfTrue="1" operator="equal">
       <formula>"w"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="729" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="729" stopIfTrue="1" operator="equal">
       <formula>"h"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="98" priority="728" stopIfTrue="1" operator="equal">
@@ -20072,7 +20092,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29:W29 C31:W31 C33:W33 C35:W35 C37:W37 C39:W39">
-    <cfRule type="expression" dxfId="94" priority="710" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="710" stopIfTrue="1">
       <formula>AND(ISNUMBER(C29),COUNTIF(Feiertage,DATE(Planungsjahr,5,C29))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="94" priority="711" stopIfTrue="1">
@@ -20080,7 +20100,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C45:W45 C47:W47 C49:W49 C51:W51 C53:W53 C55:W55">
-    <cfRule type="expression" dxfId="92" priority="718" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="718" stopIfTrue="1">
       <formula>AND(ISNUMBER(C45),COUNTIF(Feiertage,DATE(Planungsjahr,9,C45))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="92" priority="719" stopIfTrue="1">
@@ -20093,7 +20113,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z13:AT13 Z15:AT15 Z17:AT17 Z19:AT19 Z21:AT21 Z23:AT23">
-    <cfRule type="expression" dxfId="90" priority="704" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="704" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z13),COUNTIF(Feiertage,DATE(Planungsjahr,2,Z13))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="90" priority="705" stopIfTrue="1">
@@ -20101,7 +20121,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z29:AT29 Z31:AT31 Z33:AT33 Z35:AT35 Z37:AT37 Z39:AT39">
-    <cfRule type="expression" dxfId="88" priority="712" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="712" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z29),COUNTIF(Feiertage,DATE(Planungsjahr,6,Z29))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="88" priority="713" stopIfTrue="1">
@@ -20109,11 +20129,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z45:AT45 Z47:AT47 Z49:AT49 Z51:AT51 Z53:AT53 Z55:AT55">
+    <cfRule type="expression" dxfId="142" priority="720" stopIfTrue="1">
+      <formula>AND(ISNUMBER(Z45),COUNTIF(Feiertage,DATE(Planungsjahr,10,Z45))&gt;0)</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="87" priority="721" stopIfTrue="1">
       <formula>AND(ISNUMBER(Z45),WEEKDAY(DATE(Planungsjahr,10,Z45),2)&gt;5)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="87" priority="720" stopIfTrue="1">
-      <formula>AND(ISNUMBER(Z45),COUNTIF(Feiertage,DATE(Planungsjahr,10,Z45))&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AP62:AP81">
@@ -20122,23 +20142,23 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW13:BQ13 AW15:BQ15 AW17:BQ17 AW19:BQ19 AW21:BQ21 AW23:BQ23">
+    <cfRule type="expression" dxfId="142" priority="706" stopIfTrue="1">
+      <formula>AND(ISNUMBER(AW13),COUNTIF(Feiertage,DATE(Planungsjahr,3,AW13))&gt;0)</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="83" priority="707" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW13),WEEKDAY(DATE(Planungsjahr,3,AW13),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="706" stopIfTrue="1">
-      <formula>AND(ISNUMBER(AW13),COUNTIF(Feiertage,DATE(Planungsjahr,3,AW13))&gt;0)</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW29:BQ29 AW31:BQ31 AW33:BQ33 AW35:BQ35 AW37:BQ37 AW39:BQ39">
+    <cfRule type="expression" dxfId="142" priority="714" stopIfTrue="1">
+      <formula>AND(ISNUMBER(AW29),COUNTIF(Feiertage,DATE(Planungsjahr,7,AW29))&gt;0)</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="81" priority="715" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW29),WEEKDAY(DATE(Planungsjahr,7,AW29),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="714" stopIfTrue="1">
-      <formula>AND(ISNUMBER(AW29),COUNTIF(Feiertage,DATE(Planungsjahr,7,AW29))&gt;0)</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW45:BQ45 AW47:BQ47 AW49:BQ49 AW51:BQ51 AW53:BQ53 AW55:BQ55">
-    <cfRule type="expression" dxfId="78" priority="722" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="722" stopIfTrue="1">
       <formula>AND(ISNUMBER(AW45),COUNTIF(Feiertage,DATE(Planungsjahr,11,AW45))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="78" priority="723" stopIfTrue="1">
@@ -20159,15 +20179,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT13:CN13 BT15:CN15 BT17:CN17 BT19:CN19 BT21:CN21 BT23:CN23">
+    <cfRule type="expression" dxfId="142" priority="708" stopIfTrue="1">
+      <formula>AND(ISNUMBER(BT13),COUNTIF(Feiertage,DATE(Planungsjahr,4,BT13))&gt;0)</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="74" priority="709" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT13),WEEKDAY(DATE(Planungsjahr,4,BT13),2)&gt;5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="708" stopIfTrue="1">
-      <formula>AND(ISNUMBER(BT13),COUNTIF(Feiertage,DATE(Planungsjahr,4,BT13))&gt;0)</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT29:CN29 BT31:CN31 BT33:CN33 BT35:CN35 BT37:CN37 BT39:CN39">
-    <cfRule type="expression" dxfId="71" priority="716" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="716" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT29),COUNTIF(Feiertage,DATE(Planungsjahr,8,BT29))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="71" priority="717" stopIfTrue="1">
@@ -20175,7 +20195,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BT45:CN45 BT47:CN47 BT49:CN49 BT51:CN51 BT53:CN53 BT55:CN55">
-    <cfRule type="expression" dxfId="69" priority="724" stopIfTrue="1">
+    <cfRule type="expression" dxfId="142" priority="724" stopIfTrue="1">
       <formula>AND(ISNUMBER(BT45),COUNTIF(Feiertage,DATE(Planungsjahr,12,BT45))&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="69" priority="725" stopIfTrue="1">
@@ -20202,9 +20222,9 @@
       <formula1>2000</formula1>
       <formula2>2100</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Im Kalender anzeigen (S)" prompt="Häkchen = Start Selektion dieser Maßnahme wird im Kalender markiert. Häkchen entfernen = Marker ausgeblendet (die Tabelle bleibt unverändert)." sqref="P62:P81"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Im Kalender anzeigen (I)" prompt="Häkchen = Start inhaltliche Arbeit dieser Maßnahme wird im Kalender markiert. Häkchen entfernen = Marker ausgeblendet (die Tabelle bleibt unverändert)." sqref="R62:R81"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Im Kalender anzeigen (P)" prompt="Häkchen = PAL dieser Maßnahme wird im Kalender markiert. Häkchen entfernen = Marker ausgeblendet (die Tabelle bleibt unverändert)." sqref="T62:T81"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Im Kalender anzeigen (S)" prompt="Häkchen = Start Selektion dieser Maßnahme wird im Kalender markiert. Häkchen entfernen = Marker ausgeblendet (die Tabelle bleibt unverändert)." sqref="S62:S81"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Im Kalender anzeigen (I)" prompt="Häkchen = Start inhaltliche Arbeit dieser Maßnahme wird im Kalender markiert. Häkchen entfernen = Marker ausgeblendet (die Tabelle bleibt unverändert)." sqref="T62:T81"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Im Kalender anzeigen (P)" prompt="Häkchen = PAL dieser Maßnahme wird im Kalender markiert. Häkchen entfernen = Marker ausgeblendet (die Tabelle bleibt unverändert)." sqref="U62:U81"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>

</xml_diff>